<commit_message>
Updated CAN_grids model - 2025-09-17 18:40
</commit_message>
<xml_diff>
--- a/VerveStacks_CAN_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_CAN_grids/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CAN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{67F714F1-4B35-40FA-A3BE-EF8F9B505F7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3E479B79-6CB3-49FA-91CF-5580A6C32454}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2852" uniqueCount="1470">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3300" uniqueCount="1694">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -3139,1315 +3139,1987 @@
     <t>rez_sol_001</t>
   </si>
   <si>
-    <t>elc_sol_1.0</t>
+    <t>elc_sol_001</t>
   </si>
   <si>
     <t>rez_sol_002</t>
   </si>
   <si>
-    <t>elc_sol_2.0</t>
+    <t>elc_sol_002</t>
   </si>
   <si>
     <t>rez_sol_003</t>
   </si>
   <si>
-    <t>elc_sol_3.0</t>
+    <t>elc_sol_003</t>
   </si>
   <si>
     <t>rez_sol_004</t>
   </si>
   <si>
-    <t>elc_sol_4.0</t>
+    <t>elc_sol_004</t>
   </si>
   <si>
     <t>rez_sol_005</t>
   </si>
   <si>
-    <t>elc_sol_5.0</t>
+    <t>elc_sol_005</t>
   </si>
   <si>
     <t>rez_sol_006</t>
   </si>
   <si>
-    <t>elc_sol_6.0</t>
+    <t>elc_sol_006</t>
   </si>
   <si>
     <t>rez_sol_007</t>
   </si>
   <si>
-    <t>elc_sol_7.0</t>
+    <t>elc_sol_007</t>
   </si>
   <si>
     <t>rez_sol_008</t>
   </si>
   <si>
-    <t>elc_sol_8.0</t>
+    <t>elc_sol_008</t>
   </si>
   <si>
     <t>rez_sol_009</t>
   </si>
   <si>
-    <t>elc_sol_9.0</t>
+    <t>elc_sol_009</t>
   </si>
   <si>
     <t>rez_sol_010</t>
   </si>
   <si>
-    <t>elc_sol_10.0</t>
+    <t>elc_sol_010</t>
   </si>
   <si>
     <t>rez_sol_011</t>
   </si>
   <si>
-    <t>elc_sol_11.0</t>
+    <t>elc_sol_011</t>
   </si>
   <si>
     <t>rez_sol_012</t>
   </si>
   <si>
-    <t>elc_sol_12.0</t>
+    <t>elc_sol_012</t>
   </si>
   <si>
     <t>rez_sol_013</t>
   </si>
   <si>
-    <t>elc_sol_13.0</t>
+    <t>elc_sol_013</t>
   </si>
   <si>
     <t>rez_sol_014</t>
   </si>
   <si>
-    <t>elc_sol_14.0</t>
+    <t>elc_sol_014</t>
   </si>
   <si>
     <t>rez_sol_015</t>
   </si>
   <si>
-    <t>elc_sol_15.0</t>
+    <t>elc_sol_015</t>
   </si>
   <si>
     <t>rez_sol_016</t>
   </si>
   <si>
-    <t>elc_sol_16.0</t>
+    <t>elc_sol_016</t>
   </si>
   <si>
     <t>rez_sol_017</t>
   </si>
   <si>
-    <t>elc_sol_17.0</t>
+    <t>elc_sol_017</t>
   </si>
   <si>
     <t>rez_sol_018</t>
   </si>
   <si>
-    <t>elc_sol_18.0</t>
+    <t>elc_sol_018</t>
   </si>
   <si>
     <t>rez_sol_019</t>
   </si>
   <si>
-    <t>elc_sol_19.0</t>
+    <t>elc_sol_019</t>
   </si>
   <si>
     <t>rez_sol_020</t>
   </si>
   <si>
-    <t>elc_sol_20.0</t>
+    <t>elc_sol_020</t>
   </si>
   <si>
     <t>rez_sol_021</t>
   </si>
   <si>
-    <t>elc_sol_21.0</t>
+    <t>elc_sol_021</t>
   </si>
   <si>
     <t>rez_sol_022</t>
   </si>
   <si>
-    <t>elc_sol_22.0</t>
+    <t>elc_sol_022</t>
   </si>
   <si>
     <t>rez_sol_023</t>
   </si>
   <si>
-    <t>elc_sol_23.0</t>
+    <t>elc_sol_023</t>
   </si>
   <si>
     <t>rez_sol_024</t>
   </si>
   <si>
-    <t>elc_sol_24.0</t>
+    <t>elc_sol_024</t>
   </si>
   <si>
     <t>rez_sol_025</t>
   </si>
   <si>
-    <t>elc_sol_25.0</t>
+    <t>elc_sol_025</t>
   </si>
   <si>
     <t>rez_sol_026</t>
   </si>
   <si>
-    <t>elc_sol_26.0</t>
+    <t>elc_sol_026</t>
   </si>
   <si>
     <t>rez_sol_027</t>
   </si>
   <si>
-    <t>elc_sol_27.0</t>
+    <t>elc_sol_027</t>
   </si>
   <si>
     <t>rez_sol_028</t>
   </si>
   <si>
-    <t>elc_sol_28.0</t>
+    <t>elc_sol_028</t>
   </si>
   <si>
     <t>rez_sol_029</t>
   </si>
   <si>
-    <t>elc_sol_29.0</t>
+    <t>elc_sol_029</t>
   </si>
   <si>
     <t>rez_sol_030</t>
   </si>
   <si>
-    <t>elc_sol_30.0</t>
+    <t>elc_sol_030</t>
   </si>
   <si>
     <t>rez_sol_031</t>
   </si>
   <si>
-    <t>elc_sol_31.0</t>
+    <t>elc_sol_031</t>
   </si>
   <si>
     <t>rez_sol_032</t>
   </si>
   <si>
-    <t>elc_sol_32.0</t>
+    <t>elc_sol_032</t>
   </si>
   <si>
     <t>rez_sol_033</t>
   </si>
   <si>
-    <t>elc_sol_33.0</t>
+    <t>elc_sol_033</t>
   </si>
   <si>
     <t>rez_sol_034</t>
   </si>
   <si>
-    <t>elc_sol_34.0</t>
+    <t>elc_sol_034</t>
   </si>
   <si>
     <t>rez_sol_035</t>
   </si>
   <si>
-    <t>elc_sol_35.0</t>
+    <t>elc_sol_035</t>
   </si>
   <si>
     <t>rez_sol_036</t>
   </si>
   <si>
-    <t>elc_sol_36.0</t>
+    <t>elc_sol_036</t>
   </si>
   <si>
     <t>rez_sol_037</t>
   </si>
   <si>
-    <t>elc_sol_37.0</t>
+    <t>elc_sol_037</t>
   </si>
   <si>
     <t>rez_sol_038</t>
   </si>
   <si>
-    <t>elc_sol_38.0</t>
+    <t>elc_sol_038</t>
   </si>
   <si>
     <t>rez_sol_039</t>
   </si>
   <si>
-    <t>elc_sol_39.0</t>
+    <t>elc_sol_039</t>
   </si>
   <si>
     <t>rez_sol_040</t>
   </si>
   <si>
-    <t>elc_sol_40.0</t>
+    <t>elc_sol_040</t>
   </si>
   <si>
     <t>rez_sol_041</t>
   </si>
   <si>
-    <t>elc_sol_41.0</t>
+    <t>elc_sol_041</t>
   </si>
   <si>
     <t>rez_sol_042</t>
   </si>
   <si>
-    <t>elc_sol_42.0</t>
+    <t>elc_sol_042</t>
   </si>
   <si>
     <t>rez_sol_043</t>
   </si>
   <si>
-    <t>elc_sol_43.0</t>
+    <t>elc_sol_043</t>
   </si>
   <si>
     <t>rez_sol_044</t>
   </si>
   <si>
-    <t>elc_sol_44.0</t>
+    <t>elc_sol_044</t>
   </si>
   <si>
     <t>rez_sol_045</t>
   </si>
   <si>
-    <t>elc_sol_45.0</t>
+    <t>elc_sol_045</t>
   </si>
   <si>
     <t>rez_sol_046</t>
   </si>
   <si>
-    <t>elc_sol_46.0</t>
+    <t>elc_sol_046</t>
   </si>
   <si>
     <t>rez_sol_047</t>
   </si>
   <si>
-    <t>elc_sol_47.0</t>
+    <t>elc_sol_047</t>
   </si>
   <si>
     <t>rez_sol_048</t>
   </si>
   <si>
-    <t>elc_sol_48.0</t>
+    <t>elc_sol_048</t>
   </si>
   <si>
     <t>rez_sol_049</t>
   </si>
   <si>
-    <t>elc_sol_49.0</t>
+    <t>elc_sol_049</t>
   </si>
   <si>
     <t>rez_sol_050</t>
   </si>
   <si>
-    <t>elc_sol_50.0</t>
+    <t>elc_sol_050</t>
   </si>
   <si>
     <t>rez_sol_051</t>
   </si>
   <si>
-    <t>elc_sol_51.0</t>
+    <t>elc_sol_051</t>
   </si>
   <si>
     <t>rez_sol_052</t>
   </si>
   <si>
-    <t>elc_sol_52.0</t>
+    <t>elc_sol_052</t>
   </si>
   <si>
     <t>rez_sol_053</t>
   </si>
   <si>
-    <t>elc_sol_53.0</t>
+    <t>elc_sol_053</t>
   </si>
   <si>
     <t>rez_sol_054</t>
   </si>
   <si>
-    <t>elc_sol_54.0</t>
+    <t>elc_sol_054</t>
   </si>
   <si>
     <t>rez_sol_055</t>
   </si>
   <si>
-    <t>elc_sol_55.0</t>
+    <t>elc_sol_055</t>
   </si>
   <si>
     <t>rez_sol_056</t>
   </si>
   <si>
-    <t>elc_sol_56.0</t>
+    <t>elc_sol_056</t>
   </si>
   <si>
     <t>rez_sol_057</t>
   </si>
   <si>
-    <t>elc_sol_57.0</t>
+    <t>elc_sol_057</t>
   </si>
   <si>
     <t>rez_sol_058</t>
   </si>
   <si>
-    <t>elc_sol_58.0</t>
+    <t>elc_sol_058</t>
   </si>
   <si>
     <t>rez_sol_059</t>
   </si>
   <si>
-    <t>elc_sol_59.0</t>
+    <t>elc_sol_059</t>
   </si>
   <si>
     <t>rez_sol_060</t>
   </si>
   <si>
-    <t>elc_sol_60.0</t>
+    <t>elc_sol_060</t>
   </si>
   <si>
     <t>rez_sol_061</t>
   </si>
   <si>
-    <t>elc_sol_61.0</t>
+    <t>elc_sol_061</t>
   </si>
   <si>
     <t>rez_sol_062</t>
   </si>
   <si>
-    <t>elc_sol_62.0</t>
+    <t>elc_sol_062</t>
   </si>
   <si>
     <t>rez_sol_063</t>
   </si>
   <si>
-    <t>elc_sol_63.0</t>
+    <t>elc_sol_063</t>
   </si>
   <si>
     <t>rez_sol_064</t>
   </si>
   <si>
-    <t>elc_sol_64.0</t>
+    <t>elc_sol_064</t>
   </si>
   <si>
     <t>rez_sol_065</t>
   </si>
   <si>
-    <t>elc_sol_65.0</t>
+    <t>elc_sol_065</t>
   </si>
   <si>
     <t>rez_sol_066</t>
   </si>
   <si>
-    <t>elc_sol_66.0</t>
+    <t>elc_sol_066</t>
   </si>
   <si>
     <t>rez_sol_067</t>
   </si>
   <si>
-    <t>elc_sol_67.0</t>
+    <t>elc_sol_067</t>
   </si>
   <si>
     <t>rez_sol_068</t>
   </si>
   <si>
-    <t>elc_sol_68.0</t>
+    <t>elc_sol_068</t>
   </si>
   <si>
     <t>rez_sol_069</t>
   </si>
   <si>
-    <t>elc_sol_69.0</t>
+    <t>elc_sol_069</t>
   </si>
   <si>
     <t>rez_sol_070</t>
   </si>
   <si>
-    <t>elc_sol_70.0</t>
+    <t>elc_sol_070</t>
   </si>
   <si>
     <t>rez_sol_071</t>
   </si>
   <si>
-    <t>elc_sol_71.0</t>
+    <t>elc_sol_071</t>
   </si>
   <si>
     <t>rez_sol_072</t>
   </si>
   <si>
-    <t>elc_sol_72.0</t>
+    <t>elc_sol_072</t>
   </si>
   <si>
     <t>rez_sol_073</t>
   </si>
   <si>
-    <t>elc_sol_73.0</t>
+    <t>elc_sol_073</t>
   </si>
   <si>
     <t>rez_sol_074</t>
   </si>
   <si>
-    <t>elc_sol_74.0</t>
+    <t>elc_sol_074</t>
   </si>
   <si>
     <t>rez_sol_075</t>
   </si>
   <si>
-    <t>elc_sol_75.0</t>
+    <t>elc_sol_075</t>
   </si>
   <si>
     <t>rez_sol_076</t>
   </si>
   <si>
-    <t>elc_sol_76.0</t>
+    <t>elc_sol_076</t>
   </si>
   <si>
     <t>rez_sol_077</t>
   </si>
   <si>
-    <t>elc_sol_77.0</t>
+    <t>elc_sol_077</t>
   </si>
   <si>
     <t>rez_sol_078</t>
   </si>
   <si>
-    <t>elc_sol_78.0</t>
+    <t>elc_sol_078</t>
   </si>
   <si>
     <t>rez_sol_079</t>
   </si>
   <si>
-    <t>elc_sol_79.0</t>
+    <t>elc_sol_079</t>
   </si>
   <si>
     <t>rez_sol_080</t>
   </si>
   <si>
-    <t>elc_sol_80.0</t>
+    <t>elc_sol_080</t>
   </si>
   <si>
     <t>rez_sol_081</t>
   </si>
   <si>
-    <t>elc_sol_81.0</t>
+    <t>elc_sol_081</t>
   </si>
   <si>
     <t>rez_sol_082</t>
   </si>
   <si>
-    <t>elc_sol_82.0</t>
+    <t>elc_sol_082</t>
   </si>
   <si>
     <t>rez_sol_083</t>
   </si>
   <si>
-    <t>elc_sol_83.0</t>
+    <t>elc_sol_083</t>
   </si>
   <si>
     <t>rez_sol_084</t>
   </si>
   <si>
-    <t>elc_sol_84.0</t>
+    <t>elc_sol_084</t>
   </si>
   <si>
     <t>rez_sol_085</t>
   </si>
   <si>
-    <t>elc_sol_85.0</t>
+    <t>elc_sol_085</t>
   </si>
   <si>
     <t>rez_sol_086</t>
   </si>
   <si>
-    <t>elc_sol_86.0</t>
+    <t>elc_sol_086</t>
   </si>
   <si>
     <t>rez_sol_087</t>
   </si>
   <si>
-    <t>elc_sol_87.0</t>
+    <t>elc_sol_087</t>
   </si>
   <si>
     <t>rez_sol_088</t>
   </si>
   <si>
-    <t>elc_sol_88.0</t>
+    <t>elc_sol_088</t>
   </si>
   <si>
     <t>rez_sol_089</t>
   </si>
   <si>
-    <t>elc_sol_89.0</t>
+    <t>elc_sol_089</t>
   </si>
   <si>
     <t>rez_sol_090</t>
   </si>
   <si>
-    <t>elc_sol_90.0</t>
+    <t>elc_sol_090</t>
   </si>
   <si>
     <t>rez_sol_091</t>
   </si>
   <si>
-    <t>elc_sol_91.0</t>
+    <t>elc_sol_091</t>
   </si>
   <si>
     <t>rez_sol_092</t>
   </si>
   <si>
-    <t>elc_sol_92.0</t>
+    <t>elc_sol_092</t>
   </si>
   <si>
     <t>rez_sol_093</t>
   </si>
   <si>
-    <t>elc_sol_93.0</t>
+    <t>elc_sol_093</t>
   </si>
   <si>
     <t>rez_sol_094</t>
   </si>
   <si>
-    <t>elc_sol_94.0</t>
+    <t>elc_sol_094</t>
   </si>
   <si>
     <t>rez_sol_095</t>
   </si>
   <si>
-    <t>elc_sol_95.0</t>
+    <t>elc_sol_095</t>
   </si>
   <si>
     <t>rez_sol_096</t>
   </si>
   <si>
-    <t>elc_sol_96.0</t>
+    <t>elc_sol_096</t>
   </si>
   <si>
     <t>rez_sol_097</t>
   </si>
   <si>
-    <t>elc_sol_97.0</t>
+    <t>elc_sol_097</t>
   </si>
   <si>
     <t>rez_sol_098</t>
   </si>
   <si>
-    <t>elc_sol_98.0</t>
+    <t>elc_sol_098</t>
   </si>
   <si>
     <t>rez_sol_099</t>
   </si>
   <si>
-    <t>elc_sol_99.0</t>
+    <t>elc_sol_099</t>
   </si>
   <si>
     <t>rez_sol_100</t>
   </si>
   <si>
-    <t>elc_sol_100.0</t>
+    <t>elc_sol_100</t>
   </si>
   <si>
     <t>rez_sol_101</t>
   </si>
   <si>
-    <t>elc_sol_101.0</t>
+    <t>elc_sol_101</t>
   </si>
   <si>
     <t>rez_sol_102</t>
   </si>
   <si>
-    <t>elc_sol_102.0</t>
+    <t>elc_sol_102</t>
   </si>
   <si>
     <t>rez_sol_103</t>
   </si>
   <si>
-    <t>elc_sol_103.0</t>
+    <t>elc_sol_103</t>
   </si>
   <si>
     <t>rez_sol_104</t>
   </si>
   <si>
-    <t>elc_sol_104.0</t>
+    <t>elc_sol_104</t>
   </si>
   <si>
     <t>rez_sol_105</t>
   </si>
   <si>
-    <t>elc_sol_105.0</t>
+    <t>elc_sol_105</t>
   </si>
   <si>
     <t>rez_sol_106</t>
   </si>
   <si>
-    <t>elc_sol_106.0</t>
+    <t>elc_sol_106</t>
   </si>
   <si>
     <t>rez_sol_107</t>
   </si>
   <si>
-    <t>elc_sol_107.0</t>
+    <t>elc_sol_107</t>
   </si>
   <si>
     <t>rez_sol_108</t>
   </si>
   <si>
-    <t>elc_sol_108.0</t>
+    <t>elc_sol_108</t>
   </si>
   <si>
     <t>rez_sol_109</t>
   </si>
   <si>
-    <t>elc_sol_109.0</t>
+    <t>elc_sol_109</t>
   </si>
   <si>
     <t>rez_sol_110</t>
   </si>
   <si>
-    <t>elc_sol_110.0</t>
+    <t>elc_sol_110</t>
   </si>
   <si>
     <t>rez_sol_111</t>
   </si>
   <si>
-    <t>elc_sol_111.0</t>
+    <t>elc_sol_111</t>
   </si>
   <si>
     <t>rez_sol_112</t>
   </si>
   <si>
-    <t>elc_sol_112.0</t>
+    <t>elc_sol_112</t>
+  </si>
+  <si>
+    <t>rez_won_001</t>
+  </si>
+  <si>
+    <t>elc_won_001</t>
+  </si>
+  <si>
+    <t>rez_won_002</t>
+  </si>
+  <si>
+    <t>elc_won_002</t>
+  </si>
+  <si>
+    <t>rez_won_003</t>
+  </si>
+  <si>
+    <t>elc_won_003</t>
+  </si>
+  <si>
+    <t>rez_won_004</t>
+  </si>
+  <si>
+    <t>elc_won_004</t>
+  </si>
+  <si>
+    <t>rez_won_005</t>
+  </si>
+  <si>
+    <t>elc_won_005</t>
+  </si>
+  <si>
+    <t>rez_won_006</t>
+  </si>
+  <si>
+    <t>elc_won_006</t>
+  </si>
+  <si>
+    <t>rez_won_007</t>
+  </si>
+  <si>
+    <t>elc_won_007</t>
+  </si>
+  <si>
+    <t>rez_won_008</t>
+  </si>
+  <si>
+    <t>elc_won_008</t>
+  </si>
+  <si>
+    <t>rez_won_009</t>
+  </si>
+  <si>
+    <t>elc_won_009</t>
+  </si>
+  <si>
+    <t>rez_won_010</t>
+  </si>
+  <si>
+    <t>elc_won_010</t>
+  </si>
+  <si>
+    <t>rez_won_011</t>
+  </si>
+  <si>
+    <t>elc_won_011</t>
+  </si>
+  <si>
+    <t>rez_won_012</t>
+  </si>
+  <si>
+    <t>elc_won_012</t>
+  </si>
+  <si>
+    <t>rez_won_013</t>
+  </si>
+  <si>
+    <t>elc_won_013</t>
+  </si>
+  <si>
+    <t>rez_won_014</t>
+  </si>
+  <si>
+    <t>elc_won_014</t>
+  </si>
+  <si>
+    <t>rez_won_015</t>
+  </si>
+  <si>
+    <t>elc_won_015</t>
+  </si>
+  <si>
+    <t>rez_won_016</t>
+  </si>
+  <si>
+    <t>elc_won_016</t>
+  </si>
+  <si>
+    <t>rez_won_017</t>
+  </si>
+  <si>
+    <t>elc_won_017</t>
+  </si>
+  <si>
+    <t>rez_won_018</t>
+  </si>
+  <si>
+    <t>elc_won_018</t>
+  </si>
+  <si>
+    <t>rez_won_019</t>
+  </si>
+  <si>
+    <t>elc_won_019</t>
+  </si>
+  <si>
+    <t>rez_won_020</t>
+  </si>
+  <si>
+    <t>elc_won_020</t>
+  </si>
+  <si>
+    <t>rez_won_021</t>
+  </si>
+  <si>
+    <t>elc_won_021</t>
+  </si>
+  <si>
+    <t>rez_won_022</t>
+  </si>
+  <si>
+    <t>elc_won_022</t>
+  </si>
+  <si>
+    <t>rez_won_023</t>
+  </si>
+  <si>
+    <t>elc_won_023</t>
+  </si>
+  <si>
+    <t>rez_won_024</t>
+  </si>
+  <si>
+    <t>elc_won_024</t>
+  </si>
+  <si>
+    <t>rez_won_025</t>
+  </si>
+  <si>
+    <t>elc_won_025</t>
+  </si>
+  <si>
+    <t>rez_won_026</t>
+  </si>
+  <si>
+    <t>elc_won_026</t>
+  </si>
+  <si>
+    <t>rez_won_027</t>
+  </si>
+  <si>
+    <t>elc_won_027</t>
+  </si>
+  <si>
+    <t>rez_won_028</t>
+  </si>
+  <si>
+    <t>elc_won_028</t>
+  </si>
+  <si>
+    <t>rez_won_029</t>
+  </si>
+  <si>
+    <t>elc_won_029</t>
+  </si>
+  <si>
+    <t>rez_won_030</t>
+  </si>
+  <si>
+    <t>elc_won_030</t>
+  </si>
+  <si>
+    <t>rez_won_031</t>
+  </si>
+  <si>
+    <t>elc_won_031</t>
+  </si>
+  <si>
+    <t>rez_won_032</t>
+  </si>
+  <si>
+    <t>elc_won_032</t>
+  </si>
+  <si>
+    <t>rez_won_033</t>
+  </si>
+  <si>
+    <t>elc_won_033</t>
+  </si>
+  <si>
+    <t>rez_won_034</t>
+  </si>
+  <si>
+    <t>elc_won_034</t>
+  </si>
+  <si>
+    <t>rez_won_035</t>
+  </si>
+  <si>
+    <t>elc_won_035</t>
+  </si>
+  <si>
+    <t>rez_won_036</t>
+  </si>
+  <si>
+    <t>elc_won_036</t>
+  </si>
+  <si>
+    <t>rez_won_037</t>
+  </si>
+  <si>
+    <t>elc_won_037</t>
+  </si>
+  <si>
+    <t>rez_won_038</t>
+  </si>
+  <si>
+    <t>elc_won_038</t>
+  </si>
+  <si>
+    <t>rez_won_039</t>
+  </si>
+  <si>
+    <t>elc_won_039</t>
+  </si>
+  <si>
+    <t>rez_won_040</t>
+  </si>
+  <si>
+    <t>elc_won_040</t>
+  </si>
+  <si>
+    <t>rez_won_041</t>
+  </si>
+  <si>
+    <t>elc_won_041</t>
+  </si>
+  <si>
+    <t>rez_won_042</t>
+  </si>
+  <si>
+    <t>elc_won_042</t>
+  </si>
+  <si>
+    <t>rez_won_043</t>
+  </si>
+  <si>
+    <t>elc_won_043</t>
+  </si>
+  <si>
+    <t>rez_won_044</t>
+  </si>
+  <si>
+    <t>elc_won_044</t>
+  </si>
+  <si>
+    <t>rez_won_045</t>
+  </si>
+  <si>
+    <t>elc_won_045</t>
+  </si>
+  <si>
+    <t>rez_won_046</t>
+  </si>
+  <si>
+    <t>elc_won_046</t>
+  </si>
+  <si>
+    <t>rez_won_047</t>
+  </si>
+  <si>
+    <t>elc_won_047</t>
+  </si>
+  <si>
+    <t>rez_won_048</t>
+  </si>
+  <si>
+    <t>elc_won_048</t>
+  </si>
+  <si>
+    <t>rez_won_049</t>
+  </si>
+  <si>
+    <t>elc_won_049</t>
+  </si>
+  <si>
+    <t>rez_won_050</t>
+  </si>
+  <si>
+    <t>elc_won_050</t>
+  </si>
+  <si>
+    <t>rez_won_051</t>
+  </si>
+  <si>
+    <t>elc_won_051</t>
+  </si>
+  <si>
+    <t>rez_won_052</t>
+  </si>
+  <si>
+    <t>elc_won_052</t>
+  </si>
+  <si>
+    <t>rez_won_053</t>
+  </si>
+  <si>
+    <t>elc_won_053</t>
+  </si>
+  <si>
+    <t>rez_won_054</t>
+  </si>
+  <si>
+    <t>elc_won_054</t>
+  </si>
+  <si>
+    <t>rez_won_055</t>
+  </si>
+  <si>
+    <t>elc_won_055</t>
+  </si>
+  <si>
+    <t>rez_won_056</t>
+  </si>
+  <si>
+    <t>elc_won_056</t>
+  </si>
+  <si>
+    <t>rez_won_057</t>
+  </si>
+  <si>
+    <t>elc_won_057</t>
+  </si>
+  <si>
+    <t>rez_won_058</t>
+  </si>
+  <si>
+    <t>elc_won_058</t>
+  </si>
+  <si>
+    <t>rez_won_059</t>
+  </si>
+  <si>
+    <t>elc_won_059</t>
+  </si>
+  <si>
+    <t>rez_won_060</t>
+  </si>
+  <si>
+    <t>elc_won_060</t>
+  </si>
+  <si>
+    <t>rez_won_061</t>
+  </si>
+  <si>
+    <t>elc_won_061</t>
+  </si>
+  <si>
+    <t>rez_won_062</t>
+  </si>
+  <si>
+    <t>elc_won_062</t>
+  </si>
+  <si>
+    <t>rez_won_063</t>
+  </si>
+  <si>
+    <t>elc_won_063</t>
+  </si>
+  <si>
+    <t>rez_won_064</t>
+  </si>
+  <si>
+    <t>elc_won_064</t>
+  </si>
+  <si>
+    <t>rez_won_065</t>
+  </si>
+  <si>
+    <t>elc_won_065</t>
+  </si>
+  <si>
+    <t>rez_won_066</t>
+  </si>
+  <si>
+    <t>elc_won_066</t>
+  </si>
+  <si>
+    <t>rez_won_067</t>
+  </si>
+  <si>
+    <t>elc_won_067</t>
+  </si>
+  <si>
+    <t>rez_won_068</t>
+  </si>
+  <si>
+    <t>elc_won_068</t>
+  </si>
+  <si>
+    <t>rez_won_069</t>
+  </si>
+  <si>
+    <t>elc_won_069</t>
+  </si>
+  <si>
+    <t>rez_won_070</t>
+  </si>
+  <si>
+    <t>elc_won_070</t>
+  </si>
+  <si>
+    <t>rez_won_071</t>
+  </si>
+  <si>
+    <t>elc_won_071</t>
+  </si>
+  <si>
+    <t>rez_won_072</t>
+  </si>
+  <si>
+    <t>elc_won_072</t>
+  </si>
+  <si>
+    <t>rez_won_073</t>
+  </si>
+  <si>
+    <t>elc_won_073</t>
+  </si>
+  <si>
+    <t>rez_won_074</t>
+  </si>
+  <si>
+    <t>elc_won_074</t>
+  </si>
+  <si>
+    <t>rez_won_075</t>
+  </si>
+  <si>
+    <t>elc_won_075</t>
+  </si>
+  <si>
+    <t>rez_won_076</t>
+  </si>
+  <si>
+    <t>elc_won_076</t>
+  </si>
+  <si>
+    <t>rez_won_077</t>
+  </si>
+  <si>
+    <t>elc_won_077</t>
+  </si>
+  <si>
+    <t>rez_won_078</t>
+  </si>
+  <si>
+    <t>elc_won_078</t>
+  </si>
+  <si>
+    <t>rez_won_079</t>
+  </si>
+  <si>
+    <t>elc_won_079</t>
+  </si>
+  <si>
+    <t>rez_won_080</t>
+  </si>
+  <si>
+    <t>elc_won_080</t>
+  </si>
+  <si>
+    <t>rez_won_081</t>
+  </si>
+  <si>
+    <t>elc_won_081</t>
+  </si>
+  <si>
+    <t>rez_won_082</t>
+  </si>
+  <si>
+    <t>elc_won_082</t>
+  </si>
+  <si>
+    <t>rez_won_083</t>
+  </si>
+  <si>
+    <t>elc_won_083</t>
+  </si>
+  <si>
+    <t>rez_won_084</t>
+  </si>
+  <si>
+    <t>elc_won_084</t>
+  </si>
+  <si>
+    <t>rez_won_085</t>
+  </si>
+  <si>
+    <t>elc_won_085</t>
+  </si>
+  <si>
+    <t>rez_won_086</t>
+  </si>
+  <si>
+    <t>elc_won_086</t>
+  </si>
+  <si>
+    <t>rez_won_087</t>
+  </si>
+  <si>
+    <t>elc_won_087</t>
+  </si>
+  <si>
+    <t>rez_won_088</t>
+  </si>
+  <si>
+    <t>elc_won_088</t>
+  </si>
+  <si>
+    <t>rez_won_089</t>
+  </si>
+  <si>
+    <t>elc_won_089</t>
+  </si>
+  <si>
+    <t>rez_won_090</t>
+  </si>
+  <si>
+    <t>elc_won_090</t>
+  </si>
+  <si>
+    <t>rez_won_091</t>
+  </si>
+  <si>
+    <t>elc_won_091</t>
+  </si>
+  <si>
+    <t>rez_won_092</t>
+  </si>
+  <si>
+    <t>elc_won_092</t>
+  </si>
+  <si>
+    <t>rez_won_093</t>
+  </si>
+  <si>
+    <t>elc_won_093</t>
+  </si>
+  <si>
+    <t>rez_won_094</t>
+  </si>
+  <si>
+    <t>elc_won_094</t>
+  </si>
+  <si>
+    <t>rez_won_095</t>
+  </si>
+  <si>
+    <t>elc_won_095</t>
+  </si>
+  <si>
+    <t>rez_won_096</t>
+  </si>
+  <si>
+    <t>elc_won_096</t>
+  </si>
+  <si>
+    <t>rez_won_097</t>
+  </si>
+  <si>
+    <t>elc_won_097</t>
+  </si>
+  <si>
+    <t>rez_won_098</t>
+  </si>
+  <si>
+    <t>elc_won_098</t>
+  </si>
+  <si>
+    <t>rez_won_099</t>
+  </si>
+  <si>
+    <t>elc_won_099</t>
+  </si>
+  <si>
+    <t>rez_won_100</t>
+  </si>
+  <si>
+    <t>elc_won_100</t>
+  </si>
+  <si>
+    <t>rez_won_101</t>
+  </si>
+  <si>
+    <t>elc_won_101</t>
+  </si>
+  <si>
+    <t>rez_won_102</t>
+  </si>
+  <si>
+    <t>elc_won_102</t>
+  </si>
+  <si>
+    <t>rez_won_103</t>
+  </si>
+  <si>
+    <t>elc_won_103</t>
+  </si>
+  <si>
+    <t>rez_won_104</t>
+  </si>
+  <si>
+    <t>elc_won_104</t>
+  </si>
+  <si>
+    <t>rez_won_105</t>
+  </si>
+  <si>
+    <t>elc_won_105</t>
+  </si>
+  <si>
+    <t>rez_won_106</t>
+  </si>
+  <si>
+    <t>elc_won_106</t>
+  </si>
+  <si>
+    <t>rez_won_107</t>
+  </si>
+  <si>
+    <t>elc_won_107</t>
+  </si>
+  <si>
+    <t>rez_won_108</t>
+  </si>
+  <si>
+    <t>elc_won_108</t>
+  </si>
+  <si>
+    <t>rez_won_109</t>
+  </si>
+  <si>
+    <t>elc_won_109</t>
+  </si>
+  <si>
+    <t>rez_won_110</t>
+  </si>
+  <si>
+    <t>elc_won_110</t>
+  </si>
+  <si>
+    <t>rez_won_111</t>
+  </si>
+  <si>
+    <t>elc_won_111</t>
+  </si>
+  <si>
+    <t>rez_won_112</t>
+  </si>
+  <si>
+    <t>elc_won_112</t>
   </si>
   <si>
     <t>rez_wof_001</t>
   </si>
   <si>
-    <t>elc_wof_1.0</t>
+    <t>elc_wof_001</t>
   </si>
   <si>
     <t>rez_wof_002</t>
   </si>
   <si>
-    <t>elc_wof_2.0</t>
+    <t>elc_wof_002</t>
   </si>
   <si>
     <t>rez_wof_003</t>
   </si>
   <si>
-    <t>elc_wof_3.0</t>
+    <t>elc_wof_003</t>
   </si>
   <si>
     <t>rez_wof_004</t>
   </si>
   <si>
-    <t>elc_wof_4.0</t>
+    <t>elc_wof_004</t>
   </si>
   <si>
     <t>rez_wof_005</t>
   </si>
   <si>
-    <t>elc_wof_5.0</t>
+    <t>elc_wof_005</t>
   </si>
   <si>
     <t>rez_wof_006</t>
   </si>
   <si>
-    <t>elc_wof_6.0</t>
+    <t>elc_wof_006</t>
   </si>
   <si>
     <t>rez_wof_007</t>
   </si>
   <si>
-    <t>elc_wof_7.0</t>
+    <t>elc_wof_007</t>
   </si>
   <si>
     <t>rez_wof_008</t>
   </si>
   <si>
-    <t>elc_wof_8.0</t>
+    <t>elc_wof_008</t>
   </si>
   <si>
     <t>rez_wof_009</t>
   </si>
   <si>
-    <t>elc_wof_9.0</t>
+    <t>elc_wof_009</t>
   </si>
   <si>
     <t>rez_wof_010</t>
   </si>
   <si>
-    <t>elc_wof_10.0</t>
+    <t>elc_wof_010</t>
   </si>
   <si>
     <t>rez_wof_011</t>
   </si>
   <si>
-    <t>elc_wof_11.0</t>
+    <t>elc_wof_011</t>
   </si>
   <si>
     <t>rez_wof_012</t>
   </si>
   <si>
-    <t>elc_wof_12.0</t>
+    <t>elc_wof_012</t>
   </si>
   <si>
     <t>rez_wof_013</t>
   </si>
   <si>
-    <t>elc_wof_13.0</t>
+    <t>elc_wof_013</t>
   </si>
   <si>
     <t>rez_wof_014</t>
   </si>
   <si>
-    <t>elc_wof_14.0</t>
+    <t>elc_wof_014</t>
   </si>
   <si>
     <t>rez_wof_015</t>
   </si>
   <si>
-    <t>elc_wof_15.0</t>
+    <t>elc_wof_015</t>
   </si>
   <si>
     <t>rez_wof_016</t>
   </si>
   <si>
-    <t>elc_wof_16.0</t>
+    <t>elc_wof_016</t>
   </si>
   <si>
     <t>rez_wof_017</t>
   </si>
   <si>
-    <t>elc_wof_17.0</t>
+    <t>elc_wof_017</t>
   </si>
   <si>
     <t>rez_wof_018</t>
   </si>
   <si>
-    <t>elc_wof_18.0</t>
+    <t>elc_wof_018</t>
   </si>
   <si>
     <t>rez_wof_019</t>
   </si>
   <si>
-    <t>elc_wof_19.0</t>
+    <t>elc_wof_019</t>
   </si>
   <si>
     <t>rez_wof_020</t>
   </si>
   <si>
-    <t>elc_wof_20.0</t>
+    <t>elc_wof_020</t>
   </si>
   <si>
     <t>rez_wof_021</t>
   </si>
   <si>
-    <t>elc_wof_21.0</t>
+    <t>elc_wof_021</t>
   </si>
   <si>
     <t>rez_wof_022</t>
   </si>
   <si>
-    <t>elc_wof_22.0</t>
+    <t>elc_wof_022</t>
   </si>
   <si>
     <t>rez_wof_023</t>
   </si>
   <si>
-    <t>elc_wof_23.0</t>
+    <t>elc_wof_023</t>
   </si>
   <si>
     <t>rez_wof_024</t>
   </si>
   <si>
-    <t>elc_wof_24.0</t>
+    <t>elc_wof_024</t>
   </si>
   <si>
     <t>rez_wof_025</t>
   </si>
   <si>
-    <t>elc_wof_25.0</t>
+    <t>elc_wof_025</t>
   </si>
   <si>
     <t>rez_wof_026</t>
   </si>
   <si>
-    <t>elc_wof_26.0</t>
+    <t>elc_wof_026</t>
   </si>
   <si>
     <t>rez_wof_027</t>
   </si>
   <si>
-    <t>elc_wof_27.0</t>
+    <t>elc_wof_027</t>
   </si>
   <si>
     <t>rez_wof_028</t>
   </si>
   <si>
-    <t>elc_wof_28.0</t>
+    <t>elc_wof_028</t>
   </si>
   <si>
     <t>rez_wof_029</t>
   </si>
   <si>
-    <t>elc_wof_29.0</t>
+    <t>elc_wof_029</t>
   </si>
   <si>
     <t>rez_wof_030</t>
   </si>
   <si>
-    <t>elc_wof_30.0</t>
+    <t>elc_wof_030</t>
   </si>
   <si>
     <t>rez_wof_031</t>
   </si>
   <si>
-    <t>elc_wof_31.0</t>
+    <t>elc_wof_031</t>
   </si>
   <si>
     <t>rez_wof_032</t>
   </si>
   <si>
-    <t>elc_wof_32.0</t>
+    <t>elc_wof_032</t>
   </si>
   <si>
     <t>rez_wof_033</t>
   </si>
   <si>
-    <t>elc_wof_33.0</t>
+    <t>elc_wof_033</t>
   </si>
   <si>
     <t>rez_wof_034</t>
   </si>
   <si>
-    <t>elc_wof_34.0</t>
+    <t>elc_wof_034</t>
   </si>
   <si>
     <t>rez_wof_035</t>
   </si>
   <si>
-    <t>elc_wof_35.0</t>
+    <t>elc_wof_035</t>
   </si>
   <si>
     <t>rez_wof_036</t>
   </si>
   <si>
-    <t>elc_wof_36.0</t>
+    <t>elc_wof_036</t>
   </si>
   <si>
     <t>rez_wof_037</t>
   </si>
   <si>
-    <t>elc_wof_37.0</t>
+    <t>elc_wof_037</t>
   </si>
   <si>
     <t>rez_wof_038</t>
   </si>
   <si>
-    <t>elc_wof_38.0</t>
+    <t>elc_wof_038</t>
   </si>
   <si>
     <t>rez_wof_039</t>
   </si>
   <si>
-    <t>elc_wof_39.0</t>
+    <t>elc_wof_039</t>
   </si>
   <si>
     <t>rez_wof_040</t>
   </si>
   <si>
-    <t>elc_wof_40.0</t>
+    <t>elc_wof_040</t>
   </si>
   <si>
     <t>rez_wof_041</t>
   </si>
   <si>
-    <t>elc_wof_41.0</t>
+    <t>elc_wof_041</t>
   </si>
   <si>
     <t>rez_wof_042</t>
   </si>
   <si>
-    <t>elc_wof_42.0</t>
+    <t>elc_wof_042</t>
   </si>
   <si>
     <t>rez_wof_043</t>
   </si>
   <si>
-    <t>elc_wof_43.0</t>
+    <t>elc_wof_043</t>
   </si>
   <si>
     <t>rez_wof_044</t>
   </si>
   <si>
-    <t>elc_wof_44.0</t>
+    <t>elc_wof_044</t>
   </si>
   <si>
     <t>rez_wof_045</t>
   </si>
   <si>
-    <t>elc_wof_45.0</t>
+    <t>elc_wof_045</t>
   </si>
   <si>
     <t>rez_wof_046</t>
   </si>
   <si>
-    <t>elc_wof_46.0</t>
+    <t>elc_wof_046</t>
   </si>
   <si>
     <t>rez_wof_047</t>
   </si>
   <si>
-    <t>elc_wof_47.0</t>
+    <t>elc_wof_047</t>
   </si>
   <si>
     <t>rez_wof_048</t>
   </si>
   <si>
-    <t>elc_wof_48.0</t>
+    <t>elc_wof_048</t>
   </si>
   <si>
     <t>rez_wof_049</t>
   </si>
   <si>
-    <t>elc_wof_49.0</t>
+    <t>elc_wof_049</t>
   </si>
   <si>
     <t>rez_wof_050</t>
   </si>
   <si>
-    <t>elc_wof_50.0</t>
+    <t>elc_wof_050</t>
   </si>
   <si>
     <t>rez_wof_051</t>
   </si>
   <si>
-    <t>elc_wof_51.0</t>
+    <t>elc_wof_051</t>
   </si>
   <si>
     <t>rez_wof_052</t>
   </si>
   <si>
-    <t>elc_wof_52.0</t>
+    <t>elc_wof_052</t>
   </si>
   <si>
     <t>rez_wof_053</t>
   </si>
   <si>
-    <t>elc_wof_53.0</t>
+    <t>elc_wof_053</t>
   </si>
   <si>
     <t>rez_wof_054</t>
   </si>
   <si>
-    <t>elc_wof_54.0</t>
+    <t>elc_wof_054</t>
   </si>
   <si>
     <t>rez_wof_055</t>
   </si>
   <si>
-    <t>elc_wof_55.0</t>
+    <t>elc_wof_055</t>
   </si>
   <si>
     <t>rez_wof_056</t>
   </si>
   <si>
-    <t>elc_wof_56.0</t>
+    <t>elc_wof_056</t>
   </si>
   <si>
     <t>rez_wof_057</t>
   </si>
   <si>
-    <t>elc_wof_57.0</t>
+    <t>elc_wof_057</t>
   </si>
   <si>
     <t>rez_wof_058</t>
   </si>
   <si>
-    <t>elc_wof_58.0</t>
+    <t>elc_wof_058</t>
   </si>
   <si>
     <t>rez_wof_059</t>
   </si>
   <si>
-    <t>elc_wof_59.0</t>
+    <t>elc_wof_059</t>
   </si>
   <si>
     <t>rez_wof_060</t>
   </si>
   <si>
-    <t>elc_wof_60.0</t>
+    <t>elc_wof_060</t>
   </si>
   <si>
     <t>rez_wof_061</t>
   </si>
   <si>
-    <t>elc_wof_61.0</t>
+    <t>elc_wof_061</t>
   </si>
   <si>
     <t>rez_wof_062</t>
   </si>
   <si>
-    <t>elc_wof_62.0</t>
+    <t>elc_wof_062</t>
   </si>
   <si>
     <t>rez_wof_063</t>
   </si>
   <si>
-    <t>elc_wof_63.0</t>
+    <t>elc_wof_063</t>
   </si>
   <si>
     <t>rez_wof_064</t>
   </si>
   <si>
-    <t>elc_wof_64.0</t>
+    <t>elc_wof_064</t>
   </si>
   <si>
     <t>rez_wof_065</t>
   </si>
   <si>
-    <t>elc_wof_65.0</t>
+    <t>elc_wof_065</t>
   </si>
   <si>
     <t>rez_wof_066</t>
   </si>
   <si>
-    <t>elc_wof_66.0</t>
+    <t>elc_wof_066</t>
   </si>
   <si>
     <t>rez_wof_067</t>
   </si>
   <si>
-    <t>elc_wof_67.0</t>
+    <t>elc_wof_067</t>
   </si>
   <si>
     <t>rez_wof_068</t>
   </si>
   <si>
-    <t>elc_wof_68.0</t>
+    <t>elc_wof_068</t>
   </si>
   <si>
     <t>rez_wof_069</t>
   </si>
   <si>
-    <t>elc_wof_69.0</t>
+    <t>elc_wof_069</t>
   </si>
   <si>
     <t>rez_wof_070</t>
   </si>
   <si>
-    <t>elc_wof_70.0</t>
+    <t>elc_wof_070</t>
   </si>
   <si>
     <t>rez_wof_071</t>
   </si>
   <si>
-    <t>elc_wof_71.0</t>
+    <t>elc_wof_071</t>
   </si>
   <si>
     <t>rez_wof_072</t>
   </si>
   <si>
-    <t>elc_wof_72.0</t>
+    <t>elc_wof_072</t>
   </si>
   <si>
     <t>rez_wof_073</t>
   </si>
   <si>
-    <t>elc_wof_73.0</t>
+    <t>elc_wof_073</t>
   </si>
   <si>
     <t>rez_wof_074</t>
   </si>
   <si>
-    <t>elc_wof_74.0</t>
+    <t>elc_wof_074</t>
   </si>
   <si>
     <t>rez_wof_075</t>
   </si>
   <si>
-    <t>elc_wof_75.0</t>
+    <t>elc_wof_075</t>
   </si>
   <si>
     <t>rez_wof_076</t>
   </si>
   <si>
-    <t>elc_wof_76.0</t>
+    <t>elc_wof_076</t>
   </si>
   <si>
     <t>rez_wof_077</t>
   </si>
   <si>
-    <t>elc_wof_77.0</t>
+    <t>elc_wof_077</t>
   </si>
   <si>
     <t>rez_wof_078</t>
   </si>
   <si>
-    <t>elc_wof_78.0</t>
+    <t>elc_wof_078</t>
   </si>
   <si>
     <t>rez_wof_079</t>
   </si>
   <si>
-    <t>elc_wof_79.0</t>
+    <t>elc_wof_079</t>
   </si>
   <si>
     <t>rez_wof_080</t>
   </si>
   <si>
-    <t>elc_wof_80.0</t>
+    <t>elc_wof_080</t>
   </si>
   <si>
     <t>rez_wof_081</t>
   </si>
   <si>
-    <t>elc_wof_81.0</t>
+    <t>elc_wof_081</t>
   </si>
   <si>
     <t>rez_wof_082</t>
   </si>
   <si>
-    <t>elc_wof_82.0</t>
+    <t>elc_wof_082</t>
   </si>
   <si>
     <t>rez_wof_083</t>
   </si>
   <si>
-    <t>elc_wof_83.0</t>
+    <t>elc_wof_083</t>
   </si>
   <si>
     <t>rez_wof_084</t>
   </si>
   <si>
-    <t>elc_wof_84.0</t>
+    <t>elc_wof_084</t>
   </si>
   <si>
     <t>rez_wof_085</t>
   </si>
   <si>
-    <t>elc_wof_85.0</t>
+    <t>elc_wof_085</t>
   </si>
   <si>
     <t>rez_wof_086</t>
   </si>
   <si>
-    <t>elc_wof_86.0</t>
+    <t>elc_wof_086</t>
   </si>
   <si>
     <t>rez_wof_087</t>
   </si>
   <si>
-    <t>elc_wof_87.0</t>
+    <t>elc_wof_087</t>
   </si>
   <si>
     <t>rez_wof_088</t>
   </si>
   <si>
-    <t>elc_wof_88.0</t>
+    <t>elc_wof_088</t>
   </si>
   <si>
     <t>rez_wof_089</t>
   </si>
   <si>
-    <t>elc_wof_89.0</t>
+    <t>elc_wof_089</t>
   </si>
   <si>
     <t>rez_wof_090</t>
   </si>
   <si>
-    <t>elc_wof_90.0</t>
+    <t>elc_wof_090</t>
   </si>
   <si>
     <t>rez_wof_091</t>
   </si>
   <si>
-    <t>elc_wof_91.0</t>
+    <t>elc_wof_091</t>
   </si>
   <si>
     <t>rez_wof_092</t>
   </si>
   <si>
-    <t>elc_wof_92.0</t>
+    <t>elc_wof_092</t>
   </si>
   <si>
     <t>rez_wof_093</t>
   </si>
   <si>
-    <t>elc_wof_93.0</t>
+    <t>elc_wof_093</t>
   </si>
   <si>
     <t>rez_wof_094</t>
   </si>
   <si>
-    <t>elc_wof_94.0</t>
+    <t>elc_wof_094</t>
   </si>
   <si>
     <t>rez_wof_095</t>
   </si>
   <si>
-    <t>elc_wof_95.0</t>
+    <t>elc_wof_095</t>
   </si>
   <si>
     <t>rez_wof_096</t>
   </si>
   <si>
-    <t>elc_wof_96.0</t>
+    <t>elc_wof_096</t>
   </si>
   <si>
     <t>rez_wof_097</t>
   </si>
   <si>
-    <t>elc_wof_97.0</t>
+    <t>elc_wof_097</t>
   </si>
   <si>
     <t>rez_wof_098</t>
   </si>
   <si>
-    <t>elc_wof_98.0</t>
+    <t>elc_wof_098</t>
   </si>
   <si>
     <t>rez_wof_099</t>
   </si>
   <si>
-    <t>elc_wof_99.0</t>
+    <t>elc_wof_099</t>
   </si>
   <si>
     <t>rez_wof_100</t>
   </si>
   <si>
-    <t>elc_wof_100.0</t>
+    <t>elc_wof_100</t>
   </si>
   <si>
     <t>rez_wof_101</t>
   </si>
   <si>
-    <t>elc_wof_101.0</t>
+    <t>elc_wof_101</t>
   </si>
   <si>
     <t>rez_wof_102</t>
   </si>
   <si>
-    <t>elc_wof_102.0</t>
+    <t>elc_wof_102</t>
   </si>
   <si>
     <t>rez_wof_103</t>
   </si>
   <si>
-    <t>elc_wof_103.0</t>
+    <t>elc_wof_103</t>
   </si>
   <si>
     <t>rez_wof_104</t>
   </si>
   <si>
-    <t>elc_wof_104.0</t>
+    <t>elc_wof_104</t>
   </si>
   <si>
     <t>rez_wof_105</t>
   </si>
   <si>
-    <t>elc_wof_105.0</t>
+    <t>elc_wof_105</t>
   </si>
   <si>
     <t>rez_wof_106</t>
   </si>
   <si>
-    <t>elc_wof_106.0</t>
+    <t>elc_wof_106</t>
   </si>
   <si>
     <t>rez_wof_107</t>
   </si>
   <si>
-    <t>elc_wof_107.0</t>
+    <t>elc_wof_107</t>
   </si>
 </sst>
 </file>
@@ -5285,8 +5957,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CBAE67D-9E42-47E2-B42D-0FAF227B7F41}">
-  <dimension ref="B9:E693"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88F0F5B4-89F6-4F2E-8B23-FBD0C54D6F08}">
+  <dimension ref="B9:E805"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="9" spans="2:5" x14ac:dyDescent="0.45">
@@ -14867,6 +15539,1574 @@
         <v>1469</v>
       </c>
       <c r="E693" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="694" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B694" t="s">
+        <v>1470</v>
+      </c>
+      <c r="C694" t="s">
+        <v>1471</v>
+      </c>
+      <c r="D694" t="s">
+        <v>1471</v>
+      </c>
+      <c r="E694" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="695" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B695" t="s">
+        <v>1472</v>
+      </c>
+      <c r="C695" t="s">
+        <v>1473</v>
+      </c>
+      <c r="D695" t="s">
+        <v>1473</v>
+      </c>
+      <c r="E695" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="696" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B696" t="s">
+        <v>1474</v>
+      </c>
+      <c r="C696" t="s">
+        <v>1475</v>
+      </c>
+      <c r="D696" t="s">
+        <v>1475</v>
+      </c>
+      <c r="E696" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="697" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B697" t="s">
+        <v>1476</v>
+      </c>
+      <c r="C697" t="s">
+        <v>1477</v>
+      </c>
+      <c r="D697" t="s">
+        <v>1477</v>
+      </c>
+      <c r="E697" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="698" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B698" t="s">
+        <v>1478</v>
+      </c>
+      <c r="C698" t="s">
+        <v>1479</v>
+      </c>
+      <c r="D698" t="s">
+        <v>1479</v>
+      </c>
+      <c r="E698" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="699" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B699" t="s">
+        <v>1480</v>
+      </c>
+      <c r="C699" t="s">
+        <v>1481</v>
+      </c>
+      <c r="D699" t="s">
+        <v>1481</v>
+      </c>
+      <c r="E699" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="700" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B700" t="s">
+        <v>1482</v>
+      </c>
+      <c r="C700" t="s">
+        <v>1483</v>
+      </c>
+      <c r="D700" t="s">
+        <v>1483</v>
+      </c>
+      <c r="E700" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="701" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B701" t="s">
+        <v>1484</v>
+      </c>
+      <c r="C701" t="s">
+        <v>1485</v>
+      </c>
+      <c r="D701" t="s">
+        <v>1485</v>
+      </c>
+      <c r="E701" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="702" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B702" t="s">
+        <v>1486</v>
+      </c>
+      <c r="C702" t="s">
+        <v>1487</v>
+      </c>
+      <c r="D702" t="s">
+        <v>1487</v>
+      </c>
+      <c r="E702" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="703" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B703" t="s">
+        <v>1488</v>
+      </c>
+      <c r="C703" t="s">
+        <v>1489</v>
+      </c>
+      <c r="D703" t="s">
+        <v>1489</v>
+      </c>
+      <c r="E703" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="704" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B704" t="s">
+        <v>1490</v>
+      </c>
+      <c r="C704" t="s">
+        <v>1491</v>
+      </c>
+      <c r="D704" t="s">
+        <v>1491</v>
+      </c>
+      <c r="E704" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="705" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B705" t="s">
+        <v>1492</v>
+      </c>
+      <c r="C705" t="s">
+        <v>1493</v>
+      </c>
+      <c r="D705" t="s">
+        <v>1493</v>
+      </c>
+      <c r="E705" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="706" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B706" t="s">
+        <v>1494</v>
+      </c>
+      <c r="C706" t="s">
+        <v>1495</v>
+      </c>
+      <c r="D706" t="s">
+        <v>1495</v>
+      </c>
+      <c r="E706" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="707" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B707" t="s">
+        <v>1496</v>
+      </c>
+      <c r="C707" t="s">
+        <v>1497</v>
+      </c>
+      <c r="D707" t="s">
+        <v>1497</v>
+      </c>
+      <c r="E707" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="708" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B708" t="s">
+        <v>1498</v>
+      </c>
+      <c r="C708" t="s">
+        <v>1499</v>
+      </c>
+      <c r="D708" t="s">
+        <v>1499</v>
+      </c>
+      <c r="E708" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="709" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B709" t="s">
+        <v>1500</v>
+      </c>
+      <c r="C709" t="s">
+        <v>1501</v>
+      </c>
+      <c r="D709" t="s">
+        <v>1501</v>
+      </c>
+      <c r="E709" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="710" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B710" t="s">
+        <v>1502</v>
+      </c>
+      <c r="C710" t="s">
+        <v>1503</v>
+      </c>
+      <c r="D710" t="s">
+        <v>1503</v>
+      </c>
+      <c r="E710" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="711" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B711" t="s">
+        <v>1504</v>
+      </c>
+      <c r="C711" t="s">
+        <v>1505</v>
+      </c>
+      <c r="D711" t="s">
+        <v>1505</v>
+      </c>
+      <c r="E711" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="712" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B712" t="s">
+        <v>1506</v>
+      </c>
+      <c r="C712" t="s">
+        <v>1507</v>
+      </c>
+      <c r="D712" t="s">
+        <v>1507</v>
+      </c>
+      <c r="E712" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="713" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B713" t="s">
+        <v>1508</v>
+      </c>
+      <c r="C713" t="s">
+        <v>1509</v>
+      </c>
+      <c r="D713" t="s">
+        <v>1509</v>
+      </c>
+      <c r="E713" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="714" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B714" t="s">
+        <v>1510</v>
+      </c>
+      <c r="C714" t="s">
+        <v>1511</v>
+      </c>
+      <c r="D714" t="s">
+        <v>1511</v>
+      </c>
+      <c r="E714" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="715" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B715" t="s">
+        <v>1512</v>
+      </c>
+      <c r="C715" t="s">
+        <v>1513</v>
+      </c>
+      <c r="D715" t="s">
+        <v>1513</v>
+      </c>
+      <c r="E715" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="716" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B716" t="s">
+        <v>1514</v>
+      </c>
+      <c r="C716" t="s">
+        <v>1515</v>
+      </c>
+      <c r="D716" t="s">
+        <v>1515</v>
+      </c>
+      <c r="E716" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="717" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B717" t="s">
+        <v>1516</v>
+      </c>
+      <c r="C717" t="s">
+        <v>1517</v>
+      </c>
+      <c r="D717" t="s">
+        <v>1517</v>
+      </c>
+      <c r="E717" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="718" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B718" t="s">
+        <v>1518</v>
+      </c>
+      <c r="C718" t="s">
+        <v>1519</v>
+      </c>
+      <c r="D718" t="s">
+        <v>1519</v>
+      </c>
+      <c r="E718" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="719" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B719" t="s">
+        <v>1520</v>
+      </c>
+      <c r="C719" t="s">
+        <v>1521</v>
+      </c>
+      <c r="D719" t="s">
+        <v>1521</v>
+      </c>
+      <c r="E719" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="720" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B720" t="s">
+        <v>1522</v>
+      </c>
+      <c r="C720" t="s">
+        <v>1523</v>
+      </c>
+      <c r="D720" t="s">
+        <v>1523</v>
+      </c>
+      <c r="E720" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="721" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B721" t="s">
+        <v>1524</v>
+      </c>
+      <c r="C721" t="s">
+        <v>1525</v>
+      </c>
+      <c r="D721" t="s">
+        <v>1525</v>
+      </c>
+      <c r="E721" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="722" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B722" t="s">
+        <v>1526</v>
+      </c>
+      <c r="C722" t="s">
+        <v>1527</v>
+      </c>
+      <c r="D722" t="s">
+        <v>1527</v>
+      </c>
+      <c r="E722" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="723" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B723" t="s">
+        <v>1528</v>
+      </c>
+      <c r="C723" t="s">
+        <v>1529</v>
+      </c>
+      <c r="D723" t="s">
+        <v>1529</v>
+      </c>
+      <c r="E723" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="724" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B724" t="s">
+        <v>1530</v>
+      </c>
+      <c r="C724" t="s">
+        <v>1531</v>
+      </c>
+      <c r="D724" t="s">
+        <v>1531</v>
+      </c>
+      <c r="E724" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="725" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B725" t="s">
+        <v>1532</v>
+      </c>
+      <c r="C725" t="s">
+        <v>1533</v>
+      </c>
+      <c r="D725" t="s">
+        <v>1533</v>
+      </c>
+      <c r="E725" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="726" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B726" t="s">
+        <v>1534</v>
+      </c>
+      <c r="C726" t="s">
+        <v>1535</v>
+      </c>
+      <c r="D726" t="s">
+        <v>1535</v>
+      </c>
+      <c r="E726" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="727" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B727" t="s">
+        <v>1536</v>
+      </c>
+      <c r="C727" t="s">
+        <v>1537</v>
+      </c>
+      <c r="D727" t="s">
+        <v>1537</v>
+      </c>
+      <c r="E727" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="728" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B728" t="s">
+        <v>1538</v>
+      </c>
+      <c r="C728" t="s">
+        <v>1539</v>
+      </c>
+      <c r="D728" t="s">
+        <v>1539</v>
+      </c>
+      <c r="E728" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="729" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B729" t="s">
+        <v>1540</v>
+      </c>
+      <c r="C729" t="s">
+        <v>1541</v>
+      </c>
+      <c r="D729" t="s">
+        <v>1541</v>
+      </c>
+      <c r="E729" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="730" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B730" t="s">
+        <v>1542</v>
+      </c>
+      <c r="C730" t="s">
+        <v>1543</v>
+      </c>
+      <c r="D730" t="s">
+        <v>1543</v>
+      </c>
+      <c r="E730" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="731" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B731" t="s">
+        <v>1544</v>
+      </c>
+      <c r="C731" t="s">
+        <v>1545</v>
+      </c>
+      <c r="D731" t="s">
+        <v>1545</v>
+      </c>
+      <c r="E731" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="732" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B732" t="s">
+        <v>1546</v>
+      </c>
+      <c r="C732" t="s">
+        <v>1547</v>
+      </c>
+      <c r="D732" t="s">
+        <v>1547</v>
+      </c>
+      <c r="E732" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="733" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B733" t="s">
+        <v>1548</v>
+      </c>
+      <c r="C733" t="s">
+        <v>1549</v>
+      </c>
+      <c r="D733" t="s">
+        <v>1549</v>
+      </c>
+      <c r="E733" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="734" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B734" t="s">
+        <v>1550</v>
+      </c>
+      <c r="C734" t="s">
+        <v>1551</v>
+      </c>
+      <c r="D734" t="s">
+        <v>1551</v>
+      </c>
+      <c r="E734" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="735" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B735" t="s">
+        <v>1552</v>
+      </c>
+      <c r="C735" t="s">
+        <v>1553</v>
+      </c>
+      <c r="D735" t="s">
+        <v>1553</v>
+      </c>
+      <c r="E735" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="736" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B736" t="s">
+        <v>1554</v>
+      </c>
+      <c r="C736" t="s">
+        <v>1555</v>
+      </c>
+      <c r="D736" t="s">
+        <v>1555</v>
+      </c>
+      <c r="E736" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="737" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B737" t="s">
+        <v>1556</v>
+      </c>
+      <c r="C737" t="s">
+        <v>1557</v>
+      </c>
+      <c r="D737" t="s">
+        <v>1557</v>
+      </c>
+      <c r="E737" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="738" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B738" t="s">
+        <v>1558</v>
+      </c>
+      <c r="C738" t="s">
+        <v>1559</v>
+      </c>
+      <c r="D738" t="s">
+        <v>1559</v>
+      </c>
+      <c r="E738" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="739" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B739" t="s">
+        <v>1560</v>
+      </c>
+      <c r="C739" t="s">
+        <v>1561</v>
+      </c>
+      <c r="D739" t="s">
+        <v>1561</v>
+      </c>
+      <c r="E739" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="740" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B740" t="s">
+        <v>1562</v>
+      </c>
+      <c r="C740" t="s">
+        <v>1563</v>
+      </c>
+      <c r="D740" t="s">
+        <v>1563</v>
+      </c>
+      <c r="E740" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="741" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B741" t="s">
+        <v>1564</v>
+      </c>
+      <c r="C741" t="s">
+        <v>1565</v>
+      </c>
+      <c r="D741" t="s">
+        <v>1565</v>
+      </c>
+      <c r="E741" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="742" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B742" t="s">
+        <v>1566</v>
+      </c>
+      <c r="C742" t="s">
+        <v>1567</v>
+      </c>
+      <c r="D742" t="s">
+        <v>1567</v>
+      </c>
+      <c r="E742" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="743" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B743" t="s">
+        <v>1568</v>
+      </c>
+      <c r="C743" t="s">
+        <v>1569</v>
+      </c>
+      <c r="D743" t="s">
+        <v>1569</v>
+      </c>
+      <c r="E743" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="744" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B744" t="s">
+        <v>1570</v>
+      </c>
+      <c r="C744" t="s">
+        <v>1571</v>
+      </c>
+      <c r="D744" t="s">
+        <v>1571</v>
+      </c>
+      <c r="E744" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="745" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B745" t="s">
+        <v>1572</v>
+      </c>
+      <c r="C745" t="s">
+        <v>1573</v>
+      </c>
+      <c r="D745" t="s">
+        <v>1573</v>
+      </c>
+      <c r="E745" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="746" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B746" t="s">
+        <v>1574</v>
+      </c>
+      <c r="C746" t="s">
+        <v>1575</v>
+      </c>
+      <c r="D746" t="s">
+        <v>1575</v>
+      </c>
+      <c r="E746" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="747" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B747" t="s">
+        <v>1576</v>
+      </c>
+      <c r="C747" t="s">
+        <v>1577</v>
+      </c>
+      <c r="D747" t="s">
+        <v>1577</v>
+      </c>
+      <c r="E747" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="748" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B748" t="s">
+        <v>1578</v>
+      </c>
+      <c r="C748" t="s">
+        <v>1579</v>
+      </c>
+      <c r="D748" t="s">
+        <v>1579</v>
+      </c>
+      <c r="E748" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="749" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B749" t="s">
+        <v>1580</v>
+      </c>
+      <c r="C749" t="s">
+        <v>1581</v>
+      </c>
+      <c r="D749" t="s">
+        <v>1581</v>
+      </c>
+      <c r="E749" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="750" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B750" t="s">
+        <v>1582</v>
+      </c>
+      <c r="C750" t="s">
+        <v>1583</v>
+      </c>
+      <c r="D750" t="s">
+        <v>1583</v>
+      </c>
+      <c r="E750" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="751" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B751" t="s">
+        <v>1584</v>
+      </c>
+      <c r="C751" t="s">
+        <v>1585</v>
+      </c>
+      <c r="D751" t="s">
+        <v>1585</v>
+      </c>
+      <c r="E751" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="752" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B752" t="s">
+        <v>1586</v>
+      </c>
+      <c r="C752" t="s">
+        <v>1587</v>
+      </c>
+      <c r="D752" t="s">
+        <v>1587</v>
+      </c>
+      <c r="E752" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="753" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B753" t="s">
+        <v>1588</v>
+      </c>
+      <c r="C753" t="s">
+        <v>1589</v>
+      </c>
+      <c r="D753" t="s">
+        <v>1589</v>
+      </c>
+      <c r="E753" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="754" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B754" t="s">
+        <v>1590</v>
+      </c>
+      <c r="C754" t="s">
+        <v>1591</v>
+      </c>
+      <c r="D754" t="s">
+        <v>1591</v>
+      </c>
+      <c r="E754" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="755" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B755" t="s">
+        <v>1592</v>
+      </c>
+      <c r="C755" t="s">
+        <v>1593</v>
+      </c>
+      <c r="D755" t="s">
+        <v>1593</v>
+      </c>
+      <c r="E755" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="756" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B756" t="s">
+        <v>1594</v>
+      </c>
+      <c r="C756" t="s">
+        <v>1595</v>
+      </c>
+      <c r="D756" t="s">
+        <v>1595</v>
+      </c>
+      <c r="E756" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="757" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B757" t="s">
+        <v>1596</v>
+      </c>
+      <c r="C757" t="s">
+        <v>1597</v>
+      </c>
+      <c r="D757" t="s">
+        <v>1597</v>
+      </c>
+      <c r="E757" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="758" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B758" t="s">
+        <v>1598</v>
+      </c>
+      <c r="C758" t="s">
+        <v>1599</v>
+      </c>
+      <c r="D758" t="s">
+        <v>1599</v>
+      </c>
+      <c r="E758" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="759" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B759" t="s">
+        <v>1600</v>
+      </c>
+      <c r="C759" t="s">
+        <v>1601</v>
+      </c>
+      <c r="D759" t="s">
+        <v>1601</v>
+      </c>
+      <c r="E759" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="760" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B760" t="s">
+        <v>1602</v>
+      </c>
+      <c r="C760" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D760" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E760" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="761" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B761" t="s">
+        <v>1604</v>
+      </c>
+      <c r="C761" t="s">
+        <v>1605</v>
+      </c>
+      <c r="D761" t="s">
+        <v>1605</v>
+      </c>
+      <c r="E761" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="762" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B762" t="s">
+        <v>1606</v>
+      </c>
+      <c r="C762" t="s">
+        <v>1607</v>
+      </c>
+      <c r="D762" t="s">
+        <v>1607</v>
+      </c>
+      <c r="E762" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="763" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B763" t="s">
+        <v>1608</v>
+      </c>
+      <c r="C763" t="s">
+        <v>1609</v>
+      </c>
+      <c r="D763" t="s">
+        <v>1609</v>
+      </c>
+      <c r="E763" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="764" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B764" t="s">
+        <v>1610</v>
+      </c>
+      <c r="C764" t="s">
+        <v>1611</v>
+      </c>
+      <c r="D764" t="s">
+        <v>1611</v>
+      </c>
+      <c r="E764" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="765" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B765" t="s">
+        <v>1612</v>
+      </c>
+      <c r="C765" t="s">
+        <v>1613</v>
+      </c>
+      <c r="D765" t="s">
+        <v>1613</v>
+      </c>
+      <c r="E765" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="766" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B766" t="s">
+        <v>1614</v>
+      </c>
+      <c r="C766" t="s">
+        <v>1615</v>
+      </c>
+      <c r="D766" t="s">
+        <v>1615</v>
+      </c>
+      <c r="E766" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="767" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B767" t="s">
+        <v>1616</v>
+      </c>
+      <c r="C767" t="s">
+        <v>1617</v>
+      </c>
+      <c r="D767" t="s">
+        <v>1617</v>
+      </c>
+      <c r="E767" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="768" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B768" t="s">
+        <v>1618</v>
+      </c>
+      <c r="C768" t="s">
+        <v>1619</v>
+      </c>
+      <c r="D768" t="s">
+        <v>1619</v>
+      </c>
+      <c r="E768" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="769" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B769" t="s">
+        <v>1620</v>
+      </c>
+      <c r="C769" t="s">
+        <v>1621</v>
+      </c>
+      <c r="D769" t="s">
+        <v>1621</v>
+      </c>
+      <c r="E769" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="770" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B770" t="s">
+        <v>1622</v>
+      </c>
+      <c r="C770" t="s">
+        <v>1623</v>
+      </c>
+      <c r="D770" t="s">
+        <v>1623</v>
+      </c>
+      <c r="E770" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="771" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B771" t="s">
+        <v>1624</v>
+      </c>
+      <c r="C771" t="s">
+        <v>1625</v>
+      </c>
+      <c r="D771" t="s">
+        <v>1625</v>
+      </c>
+      <c r="E771" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="772" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B772" t="s">
+        <v>1626</v>
+      </c>
+      <c r="C772" t="s">
+        <v>1627</v>
+      </c>
+      <c r="D772" t="s">
+        <v>1627</v>
+      </c>
+      <c r="E772" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="773" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B773" t="s">
+        <v>1628</v>
+      </c>
+      <c r="C773" t="s">
+        <v>1629</v>
+      </c>
+      <c r="D773" t="s">
+        <v>1629</v>
+      </c>
+      <c r="E773" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="774" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B774" t="s">
+        <v>1630</v>
+      </c>
+      <c r="C774" t="s">
+        <v>1631</v>
+      </c>
+      <c r="D774" t="s">
+        <v>1631</v>
+      </c>
+      <c r="E774" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="775" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B775" t="s">
+        <v>1632</v>
+      </c>
+      <c r="C775" t="s">
+        <v>1633</v>
+      </c>
+      <c r="D775" t="s">
+        <v>1633</v>
+      </c>
+      <c r="E775" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="776" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B776" t="s">
+        <v>1634</v>
+      </c>
+      <c r="C776" t="s">
+        <v>1635</v>
+      </c>
+      <c r="D776" t="s">
+        <v>1635</v>
+      </c>
+      <c r="E776" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="777" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B777" t="s">
+        <v>1636</v>
+      </c>
+      <c r="C777" t="s">
+        <v>1637</v>
+      </c>
+      <c r="D777" t="s">
+        <v>1637</v>
+      </c>
+      <c r="E777" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="778" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B778" t="s">
+        <v>1638</v>
+      </c>
+      <c r="C778" t="s">
+        <v>1639</v>
+      </c>
+      <c r="D778" t="s">
+        <v>1639</v>
+      </c>
+      <c r="E778" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="779" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B779" t="s">
+        <v>1640</v>
+      </c>
+      <c r="C779" t="s">
+        <v>1641</v>
+      </c>
+      <c r="D779" t="s">
+        <v>1641</v>
+      </c>
+      <c r="E779" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="780" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B780" t="s">
+        <v>1642</v>
+      </c>
+      <c r="C780" t="s">
+        <v>1643</v>
+      </c>
+      <c r="D780" t="s">
+        <v>1643</v>
+      </c>
+      <c r="E780" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="781" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B781" t="s">
+        <v>1644</v>
+      </c>
+      <c r="C781" t="s">
+        <v>1645</v>
+      </c>
+      <c r="D781" t="s">
+        <v>1645</v>
+      </c>
+      <c r="E781" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="782" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B782" t="s">
+        <v>1646</v>
+      </c>
+      <c r="C782" t="s">
+        <v>1647</v>
+      </c>
+      <c r="D782" t="s">
+        <v>1647</v>
+      </c>
+      <c r="E782" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="783" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B783" t="s">
+        <v>1648</v>
+      </c>
+      <c r="C783" t="s">
+        <v>1649</v>
+      </c>
+      <c r="D783" t="s">
+        <v>1649</v>
+      </c>
+      <c r="E783" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="784" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B784" t="s">
+        <v>1650</v>
+      </c>
+      <c r="C784" t="s">
+        <v>1651</v>
+      </c>
+      <c r="D784" t="s">
+        <v>1651</v>
+      </c>
+      <c r="E784" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="785" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B785" t="s">
+        <v>1652</v>
+      </c>
+      <c r="C785" t="s">
+        <v>1653</v>
+      </c>
+      <c r="D785" t="s">
+        <v>1653</v>
+      </c>
+      <c r="E785" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="786" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B786" t="s">
+        <v>1654</v>
+      </c>
+      <c r="C786" t="s">
+        <v>1655</v>
+      </c>
+      <c r="D786" t="s">
+        <v>1655</v>
+      </c>
+      <c r="E786" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="787" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B787" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C787" t="s">
+        <v>1657</v>
+      </c>
+      <c r="D787" t="s">
+        <v>1657</v>
+      </c>
+      <c r="E787" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="788" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B788" t="s">
+        <v>1658</v>
+      </c>
+      <c r="C788" t="s">
+        <v>1659</v>
+      </c>
+      <c r="D788" t="s">
+        <v>1659</v>
+      </c>
+      <c r="E788" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="789" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B789" t="s">
+        <v>1660</v>
+      </c>
+      <c r="C789" t="s">
+        <v>1661</v>
+      </c>
+      <c r="D789" t="s">
+        <v>1661</v>
+      </c>
+      <c r="E789" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="790" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B790" t="s">
+        <v>1662</v>
+      </c>
+      <c r="C790" t="s">
+        <v>1663</v>
+      </c>
+      <c r="D790" t="s">
+        <v>1663</v>
+      </c>
+      <c r="E790" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="791" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B791" t="s">
+        <v>1664</v>
+      </c>
+      <c r="C791" t="s">
+        <v>1665</v>
+      </c>
+      <c r="D791" t="s">
+        <v>1665</v>
+      </c>
+      <c r="E791" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="792" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B792" t="s">
+        <v>1666</v>
+      </c>
+      <c r="C792" t="s">
+        <v>1667</v>
+      </c>
+      <c r="D792" t="s">
+        <v>1667</v>
+      </c>
+      <c r="E792" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="793" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B793" t="s">
+        <v>1668</v>
+      </c>
+      <c r="C793" t="s">
+        <v>1669</v>
+      </c>
+      <c r="D793" t="s">
+        <v>1669</v>
+      </c>
+      <c r="E793" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="794" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B794" t="s">
+        <v>1670</v>
+      </c>
+      <c r="C794" t="s">
+        <v>1671</v>
+      </c>
+      <c r="D794" t="s">
+        <v>1671</v>
+      </c>
+      <c r="E794" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="795" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B795" t="s">
+        <v>1672</v>
+      </c>
+      <c r="C795" t="s">
+        <v>1673</v>
+      </c>
+      <c r="D795" t="s">
+        <v>1673</v>
+      </c>
+      <c r="E795" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="796" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B796" t="s">
+        <v>1674</v>
+      </c>
+      <c r="C796" t="s">
+        <v>1675</v>
+      </c>
+      <c r="D796" t="s">
+        <v>1675</v>
+      </c>
+      <c r="E796" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="797" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B797" t="s">
+        <v>1676</v>
+      </c>
+      <c r="C797" t="s">
+        <v>1677</v>
+      </c>
+      <c r="D797" t="s">
+        <v>1677</v>
+      </c>
+      <c r="E797" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="798" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B798" t="s">
+        <v>1678</v>
+      </c>
+      <c r="C798" t="s">
+        <v>1679</v>
+      </c>
+      <c r="D798" t="s">
+        <v>1679</v>
+      </c>
+      <c r="E798" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="799" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B799" t="s">
+        <v>1680</v>
+      </c>
+      <c r="C799" t="s">
+        <v>1681</v>
+      </c>
+      <c r="D799" t="s">
+        <v>1681</v>
+      </c>
+      <c r="E799" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="800" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B800" t="s">
+        <v>1682</v>
+      </c>
+      <c r="C800" t="s">
+        <v>1683</v>
+      </c>
+      <c r="D800" t="s">
+        <v>1683</v>
+      </c>
+      <c r="E800" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="801" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B801" t="s">
+        <v>1684</v>
+      </c>
+      <c r="C801" t="s">
+        <v>1685</v>
+      </c>
+      <c r="D801" t="s">
+        <v>1685</v>
+      </c>
+      <c r="E801" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="802" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B802" t="s">
+        <v>1686</v>
+      </c>
+      <c r="C802" t="s">
+        <v>1687</v>
+      </c>
+      <c r="D802" t="s">
+        <v>1687</v>
+      </c>
+      <c r="E802" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="803" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B803" t="s">
+        <v>1688</v>
+      </c>
+      <c r="C803" t="s">
+        <v>1689</v>
+      </c>
+      <c r="D803" t="s">
+        <v>1689</v>
+      </c>
+      <c r="E803" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="804" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B804" t="s">
+        <v>1690</v>
+      </c>
+      <c r="C804" t="s">
+        <v>1691</v>
+      </c>
+      <c r="D804" t="s">
+        <v>1691</v>
+      </c>
+      <c r="E804" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="805" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B805" t="s">
+        <v>1692</v>
+      </c>
+      <c r="C805" t="s">
+        <v>1693</v>
+      </c>
+      <c r="D805" t="s">
+        <v>1693</v>
+      </c>
+      <c r="E805" t="s">
         <v>105</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated CAN_grids model - 2025-09-19 00:56
</commit_message>
<xml_diff>
--- a/VerveStacks_CAN_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_CAN_grids/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CAN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3E479B79-6CB3-49FA-91CF-5580A6C32454}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CE97F6B3-438B-4837-90B6-C9D9FF8C41B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3136,676 +3136,676 @@
     <t>e_CA229*</t>
   </si>
   <si>
-    <t>rez_sol_001</t>
-  </si>
-  <si>
-    <t>elc_sol_001</t>
-  </si>
-  <si>
-    <t>rez_sol_002</t>
-  </si>
-  <si>
-    <t>elc_sol_002</t>
-  </si>
-  <si>
-    <t>rez_sol_003</t>
-  </si>
-  <si>
-    <t>elc_sol_003</t>
-  </si>
-  <si>
-    <t>rez_sol_004</t>
-  </si>
-  <si>
-    <t>elc_sol_004</t>
-  </si>
-  <si>
-    <t>rez_sol_005</t>
-  </si>
-  <si>
-    <t>elc_sol_005</t>
-  </si>
-  <si>
-    <t>rez_sol_006</t>
-  </si>
-  <si>
-    <t>elc_sol_006</t>
-  </si>
-  <si>
-    <t>rez_sol_007</t>
-  </si>
-  <si>
-    <t>elc_sol_007</t>
-  </si>
-  <si>
-    <t>rez_sol_008</t>
-  </si>
-  <si>
-    <t>elc_sol_008</t>
-  </si>
-  <si>
-    <t>rez_sol_009</t>
-  </si>
-  <si>
-    <t>elc_sol_009</t>
-  </si>
-  <si>
-    <t>rez_sol_010</t>
-  </si>
-  <si>
-    <t>elc_sol_010</t>
-  </si>
-  <si>
-    <t>rez_sol_011</t>
-  </si>
-  <si>
-    <t>elc_sol_011</t>
-  </si>
-  <si>
-    <t>rez_sol_012</t>
-  </si>
-  <si>
-    <t>elc_sol_012</t>
-  </si>
-  <si>
-    <t>rez_sol_013</t>
-  </si>
-  <si>
-    <t>elc_sol_013</t>
-  </si>
-  <si>
-    <t>rez_sol_014</t>
-  </si>
-  <si>
-    <t>elc_sol_014</t>
-  </si>
-  <si>
-    <t>rez_sol_015</t>
-  </si>
-  <si>
-    <t>elc_sol_015</t>
-  </si>
-  <si>
-    <t>rez_sol_016</t>
-  </si>
-  <si>
-    <t>elc_sol_016</t>
-  </si>
-  <si>
-    <t>rez_sol_017</t>
-  </si>
-  <si>
-    <t>elc_sol_017</t>
-  </si>
-  <si>
-    <t>rez_sol_018</t>
-  </si>
-  <si>
-    <t>elc_sol_018</t>
-  </si>
-  <si>
-    <t>rez_sol_019</t>
-  </si>
-  <si>
-    <t>elc_sol_019</t>
-  </si>
-  <si>
-    <t>rez_sol_020</t>
-  </si>
-  <si>
-    <t>elc_sol_020</t>
-  </si>
-  <si>
-    <t>rez_sol_021</t>
-  </si>
-  <si>
-    <t>elc_sol_021</t>
-  </si>
-  <si>
-    <t>rez_sol_022</t>
-  </si>
-  <si>
-    <t>elc_sol_022</t>
-  </si>
-  <si>
-    <t>rez_sol_023</t>
-  </si>
-  <si>
-    <t>elc_sol_023</t>
-  </si>
-  <si>
-    <t>rez_sol_024</t>
-  </si>
-  <si>
-    <t>elc_sol_024</t>
-  </si>
-  <si>
-    <t>rez_sol_025</t>
-  </si>
-  <si>
-    <t>elc_sol_025</t>
-  </si>
-  <si>
-    <t>rez_sol_026</t>
-  </si>
-  <si>
-    <t>elc_sol_026</t>
-  </si>
-  <si>
-    <t>rez_sol_027</t>
-  </si>
-  <si>
-    <t>elc_sol_027</t>
-  </si>
-  <si>
-    <t>rez_sol_028</t>
-  </si>
-  <si>
-    <t>elc_sol_028</t>
-  </si>
-  <si>
-    <t>rez_sol_029</t>
-  </si>
-  <si>
-    <t>elc_sol_029</t>
-  </si>
-  <si>
-    <t>rez_sol_030</t>
-  </si>
-  <si>
-    <t>elc_sol_030</t>
-  </si>
-  <si>
-    <t>rez_sol_031</t>
-  </si>
-  <si>
-    <t>elc_sol_031</t>
-  </si>
-  <si>
-    <t>rez_sol_032</t>
-  </si>
-  <si>
-    <t>elc_sol_032</t>
-  </si>
-  <si>
-    <t>rez_sol_033</t>
-  </si>
-  <si>
-    <t>elc_sol_033</t>
-  </si>
-  <si>
-    <t>rez_sol_034</t>
-  </si>
-  <si>
-    <t>elc_sol_034</t>
-  </si>
-  <si>
-    <t>rez_sol_035</t>
-  </si>
-  <si>
-    <t>elc_sol_035</t>
-  </si>
-  <si>
-    <t>rez_sol_036</t>
-  </si>
-  <si>
-    <t>elc_sol_036</t>
-  </si>
-  <si>
-    <t>rez_sol_037</t>
-  </si>
-  <si>
-    <t>elc_sol_037</t>
-  </si>
-  <si>
-    <t>rez_sol_038</t>
-  </si>
-  <si>
-    <t>elc_sol_038</t>
-  </si>
-  <si>
-    <t>rez_sol_039</t>
-  </si>
-  <si>
-    <t>elc_sol_039</t>
-  </si>
-  <si>
-    <t>rez_sol_040</t>
-  </si>
-  <si>
-    <t>elc_sol_040</t>
-  </si>
-  <si>
-    <t>rez_sol_041</t>
-  </si>
-  <si>
-    <t>elc_sol_041</t>
-  </si>
-  <si>
-    <t>rez_sol_042</t>
-  </si>
-  <si>
-    <t>elc_sol_042</t>
-  </si>
-  <si>
-    <t>rez_sol_043</t>
-  </si>
-  <si>
-    <t>elc_sol_043</t>
-  </si>
-  <si>
-    <t>rez_sol_044</t>
-  </si>
-  <si>
-    <t>elc_sol_044</t>
-  </si>
-  <si>
-    <t>rez_sol_045</t>
-  </si>
-  <si>
-    <t>elc_sol_045</t>
-  </si>
-  <si>
-    <t>rez_sol_046</t>
-  </si>
-  <si>
-    <t>elc_sol_046</t>
-  </si>
-  <si>
-    <t>rez_sol_047</t>
-  </si>
-  <si>
-    <t>elc_sol_047</t>
-  </si>
-  <si>
-    <t>rez_sol_048</t>
-  </si>
-  <si>
-    <t>elc_sol_048</t>
-  </si>
-  <si>
-    <t>rez_sol_049</t>
-  </si>
-  <si>
-    <t>elc_sol_049</t>
-  </si>
-  <si>
-    <t>rez_sol_050</t>
-  </si>
-  <si>
-    <t>elc_sol_050</t>
-  </si>
-  <si>
-    <t>rez_sol_051</t>
-  </si>
-  <si>
-    <t>elc_sol_051</t>
-  </si>
-  <si>
-    <t>rez_sol_052</t>
-  </si>
-  <si>
-    <t>elc_sol_052</t>
-  </si>
-  <si>
-    <t>rez_sol_053</t>
-  </si>
-  <si>
-    <t>elc_sol_053</t>
-  </si>
-  <si>
-    <t>rez_sol_054</t>
-  </si>
-  <si>
-    <t>elc_sol_054</t>
-  </si>
-  <si>
-    <t>rez_sol_055</t>
-  </si>
-  <si>
-    <t>elc_sol_055</t>
-  </si>
-  <si>
-    <t>rez_sol_056</t>
-  </si>
-  <si>
-    <t>elc_sol_056</t>
-  </si>
-  <si>
-    <t>rez_sol_057</t>
-  </si>
-  <si>
-    <t>elc_sol_057</t>
-  </si>
-  <si>
-    <t>rez_sol_058</t>
-  </si>
-  <si>
-    <t>elc_sol_058</t>
-  </si>
-  <si>
-    <t>rez_sol_059</t>
-  </si>
-  <si>
-    <t>elc_sol_059</t>
-  </si>
-  <si>
-    <t>rez_sol_060</t>
-  </si>
-  <si>
-    <t>elc_sol_060</t>
-  </si>
-  <si>
-    <t>rez_sol_061</t>
-  </si>
-  <si>
-    <t>elc_sol_061</t>
-  </si>
-  <si>
-    <t>rez_sol_062</t>
-  </si>
-  <si>
-    <t>elc_sol_062</t>
-  </si>
-  <si>
-    <t>rez_sol_063</t>
-  </si>
-  <si>
-    <t>elc_sol_063</t>
-  </si>
-  <si>
-    <t>rez_sol_064</t>
-  </si>
-  <si>
-    <t>elc_sol_064</t>
-  </si>
-  <si>
-    <t>rez_sol_065</t>
-  </si>
-  <si>
-    <t>elc_sol_065</t>
-  </si>
-  <si>
-    <t>rez_sol_066</t>
-  </si>
-  <si>
-    <t>elc_sol_066</t>
-  </si>
-  <si>
-    <t>rez_sol_067</t>
-  </si>
-  <si>
-    <t>elc_sol_067</t>
-  </si>
-  <si>
-    <t>rez_sol_068</t>
-  </si>
-  <si>
-    <t>elc_sol_068</t>
-  </si>
-  <si>
-    <t>rez_sol_069</t>
-  </si>
-  <si>
-    <t>elc_sol_069</t>
-  </si>
-  <si>
-    <t>rez_sol_070</t>
-  </si>
-  <si>
-    <t>elc_sol_070</t>
-  </si>
-  <si>
-    <t>rez_sol_071</t>
-  </si>
-  <si>
-    <t>elc_sol_071</t>
-  </si>
-  <si>
-    <t>rez_sol_072</t>
-  </si>
-  <si>
-    <t>elc_sol_072</t>
-  </si>
-  <si>
-    <t>rez_sol_073</t>
-  </si>
-  <si>
-    <t>elc_sol_073</t>
-  </si>
-  <si>
-    <t>rez_sol_074</t>
-  </si>
-  <si>
-    <t>elc_sol_074</t>
-  </si>
-  <si>
-    <t>rez_sol_075</t>
-  </si>
-  <si>
-    <t>elc_sol_075</t>
-  </si>
-  <si>
-    <t>rez_sol_076</t>
-  </si>
-  <si>
-    <t>elc_sol_076</t>
-  </si>
-  <si>
-    <t>rez_sol_077</t>
-  </si>
-  <si>
-    <t>elc_sol_077</t>
-  </si>
-  <si>
-    <t>rez_sol_078</t>
-  </si>
-  <si>
-    <t>elc_sol_078</t>
-  </si>
-  <si>
-    <t>rez_sol_079</t>
-  </si>
-  <si>
-    <t>elc_sol_079</t>
-  </si>
-  <si>
-    <t>rez_sol_080</t>
-  </si>
-  <si>
-    <t>elc_sol_080</t>
-  </si>
-  <si>
-    <t>rez_sol_081</t>
-  </si>
-  <si>
-    <t>elc_sol_081</t>
-  </si>
-  <si>
-    <t>rez_sol_082</t>
-  </si>
-  <si>
-    <t>elc_sol_082</t>
-  </si>
-  <si>
-    <t>rez_sol_083</t>
-  </si>
-  <si>
-    <t>elc_sol_083</t>
-  </si>
-  <si>
-    <t>rez_sol_084</t>
-  </si>
-  <si>
-    <t>elc_sol_084</t>
-  </si>
-  <si>
-    <t>rez_sol_085</t>
-  </si>
-  <si>
-    <t>elc_sol_085</t>
-  </si>
-  <si>
-    <t>rez_sol_086</t>
-  </si>
-  <si>
-    <t>elc_sol_086</t>
-  </si>
-  <si>
-    <t>rez_sol_087</t>
-  </si>
-  <si>
-    <t>elc_sol_087</t>
-  </si>
-  <si>
-    <t>rez_sol_088</t>
-  </si>
-  <si>
-    <t>elc_sol_088</t>
-  </si>
-  <si>
-    <t>rez_sol_089</t>
-  </si>
-  <si>
-    <t>elc_sol_089</t>
-  </si>
-  <si>
-    <t>rez_sol_090</t>
-  </si>
-  <si>
-    <t>elc_sol_090</t>
-  </si>
-  <si>
-    <t>rez_sol_091</t>
-  </si>
-  <si>
-    <t>elc_sol_091</t>
-  </si>
-  <si>
-    <t>rez_sol_092</t>
-  </si>
-  <si>
-    <t>elc_sol_092</t>
-  </si>
-  <si>
-    <t>rez_sol_093</t>
-  </si>
-  <si>
-    <t>elc_sol_093</t>
-  </si>
-  <si>
-    <t>rez_sol_094</t>
-  </si>
-  <si>
-    <t>elc_sol_094</t>
-  </si>
-  <si>
-    <t>rez_sol_095</t>
-  </si>
-  <si>
-    <t>elc_sol_095</t>
-  </si>
-  <si>
-    <t>rez_sol_096</t>
-  </si>
-  <si>
-    <t>elc_sol_096</t>
-  </si>
-  <si>
-    <t>rez_sol_097</t>
-  </si>
-  <si>
-    <t>elc_sol_097</t>
-  </si>
-  <si>
-    <t>rez_sol_098</t>
-  </si>
-  <si>
-    <t>elc_sol_098</t>
-  </si>
-  <si>
-    <t>rez_sol_099</t>
-  </si>
-  <si>
-    <t>elc_sol_099</t>
-  </si>
-  <si>
-    <t>rez_sol_100</t>
-  </si>
-  <si>
-    <t>elc_sol_100</t>
-  </si>
-  <si>
-    <t>rez_sol_101</t>
-  </si>
-  <si>
-    <t>elc_sol_101</t>
-  </si>
-  <si>
-    <t>rez_sol_102</t>
-  </si>
-  <si>
-    <t>elc_sol_102</t>
-  </si>
-  <si>
-    <t>rez_sol_103</t>
-  </si>
-  <si>
-    <t>elc_sol_103</t>
-  </si>
-  <si>
-    <t>rez_sol_104</t>
-  </si>
-  <si>
-    <t>elc_sol_104</t>
-  </si>
-  <si>
-    <t>rez_sol_105</t>
-  </si>
-  <si>
-    <t>elc_sol_105</t>
-  </si>
-  <si>
-    <t>rez_sol_106</t>
-  </si>
-  <si>
-    <t>elc_sol_106</t>
-  </si>
-  <si>
-    <t>rez_sol_107</t>
-  </si>
-  <si>
-    <t>elc_sol_107</t>
-  </si>
-  <si>
-    <t>rez_sol_108</t>
-  </si>
-  <si>
-    <t>elc_sol_108</t>
-  </si>
-  <si>
-    <t>rez_sol_109</t>
-  </si>
-  <si>
-    <t>elc_sol_109</t>
-  </si>
-  <si>
-    <t>rez_sol_110</t>
-  </si>
-  <si>
-    <t>elc_sol_110</t>
-  </si>
-  <si>
-    <t>rez_sol_111</t>
-  </si>
-  <si>
-    <t>elc_sol_111</t>
-  </si>
-  <si>
-    <t>rez_sol_112</t>
-  </si>
-  <si>
-    <t>elc_sol_112</t>
+    <t>rez_spv_001</t>
+  </si>
+  <si>
+    <t>elc_spv_001</t>
+  </si>
+  <si>
+    <t>rez_spv_002</t>
+  </si>
+  <si>
+    <t>elc_spv_002</t>
+  </si>
+  <si>
+    <t>rez_spv_003</t>
+  </si>
+  <si>
+    <t>elc_spv_003</t>
+  </si>
+  <si>
+    <t>rez_spv_004</t>
+  </si>
+  <si>
+    <t>elc_spv_004</t>
+  </si>
+  <si>
+    <t>rez_spv_005</t>
+  </si>
+  <si>
+    <t>elc_spv_005</t>
+  </si>
+  <si>
+    <t>rez_spv_006</t>
+  </si>
+  <si>
+    <t>elc_spv_006</t>
+  </si>
+  <si>
+    <t>rez_spv_007</t>
+  </si>
+  <si>
+    <t>elc_spv_007</t>
+  </si>
+  <si>
+    <t>rez_spv_008</t>
+  </si>
+  <si>
+    <t>elc_spv_008</t>
+  </si>
+  <si>
+    <t>rez_spv_009</t>
+  </si>
+  <si>
+    <t>elc_spv_009</t>
+  </si>
+  <si>
+    <t>rez_spv_010</t>
+  </si>
+  <si>
+    <t>elc_spv_010</t>
+  </si>
+  <si>
+    <t>rez_spv_011</t>
+  </si>
+  <si>
+    <t>elc_spv_011</t>
+  </si>
+  <si>
+    <t>rez_spv_012</t>
+  </si>
+  <si>
+    <t>elc_spv_012</t>
+  </si>
+  <si>
+    <t>rez_spv_013</t>
+  </si>
+  <si>
+    <t>elc_spv_013</t>
+  </si>
+  <si>
+    <t>rez_spv_014</t>
+  </si>
+  <si>
+    <t>elc_spv_014</t>
+  </si>
+  <si>
+    <t>rez_spv_015</t>
+  </si>
+  <si>
+    <t>elc_spv_015</t>
+  </si>
+  <si>
+    <t>rez_spv_016</t>
+  </si>
+  <si>
+    <t>elc_spv_016</t>
+  </si>
+  <si>
+    <t>rez_spv_017</t>
+  </si>
+  <si>
+    <t>elc_spv_017</t>
+  </si>
+  <si>
+    <t>rez_spv_018</t>
+  </si>
+  <si>
+    <t>elc_spv_018</t>
+  </si>
+  <si>
+    <t>rez_spv_019</t>
+  </si>
+  <si>
+    <t>elc_spv_019</t>
+  </si>
+  <si>
+    <t>rez_spv_020</t>
+  </si>
+  <si>
+    <t>elc_spv_020</t>
+  </si>
+  <si>
+    <t>rez_spv_021</t>
+  </si>
+  <si>
+    <t>elc_spv_021</t>
+  </si>
+  <si>
+    <t>rez_spv_022</t>
+  </si>
+  <si>
+    <t>elc_spv_022</t>
+  </si>
+  <si>
+    <t>rez_spv_023</t>
+  </si>
+  <si>
+    <t>elc_spv_023</t>
+  </si>
+  <si>
+    <t>rez_spv_024</t>
+  </si>
+  <si>
+    <t>elc_spv_024</t>
+  </si>
+  <si>
+    <t>rez_spv_025</t>
+  </si>
+  <si>
+    <t>elc_spv_025</t>
+  </si>
+  <si>
+    <t>rez_spv_026</t>
+  </si>
+  <si>
+    <t>elc_spv_026</t>
+  </si>
+  <si>
+    <t>rez_spv_027</t>
+  </si>
+  <si>
+    <t>elc_spv_027</t>
+  </si>
+  <si>
+    <t>rez_spv_028</t>
+  </si>
+  <si>
+    <t>elc_spv_028</t>
+  </si>
+  <si>
+    <t>rez_spv_029</t>
+  </si>
+  <si>
+    <t>elc_spv_029</t>
+  </si>
+  <si>
+    <t>rez_spv_030</t>
+  </si>
+  <si>
+    <t>elc_spv_030</t>
+  </si>
+  <si>
+    <t>rez_spv_031</t>
+  </si>
+  <si>
+    <t>elc_spv_031</t>
+  </si>
+  <si>
+    <t>rez_spv_032</t>
+  </si>
+  <si>
+    <t>elc_spv_032</t>
+  </si>
+  <si>
+    <t>rez_spv_033</t>
+  </si>
+  <si>
+    <t>elc_spv_033</t>
+  </si>
+  <si>
+    <t>rez_spv_034</t>
+  </si>
+  <si>
+    <t>elc_spv_034</t>
+  </si>
+  <si>
+    <t>rez_spv_035</t>
+  </si>
+  <si>
+    <t>elc_spv_035</t>
+  </si>
+  <si>
+    <t>rez_spv_036</t>
+  </si>
+  <si>
+    <t>elc_spv_036</t>
+  </si>
+  <si>
+    <t>rez_spv_037</t>
+  </si>
+  <si>
+    <t>elc_spv_037</t>
+  </si>
+  <si>
+    <t>rez_spv_038</t>
+  </si>
+  <si>
+    <t>elc_spv_038</t>
+  </si>
+  <si>
+    <t>rez_spv_039</t>
+  </si>
+  <si>
+    <t>elc_spv_039</t>
+  </si>
+  <si>
+    <t>rez_spv_040</t>
+  </si>
+  <si>
+    <t>elc_spv_040</t>
+  </si>
+  <si>
+    <t>rez_spv_041</t>
+  </si>
+  <si>
+    <t>elc_spv_041</t>
+  </si>
+  <si>
+    <t>rez_spv_042</t>
+  </si>
+  <si>
+    <t>elc_spv_042</t>
+  </si>
+  <si>
+    <t>rez_spv_043</t>
+  </si>
+  <si>
+    <t>elc_spv_043</t>
+  </si>
+  <si>
+    <t>rez_spv_044</t>
+  </si>
+  <si>
+    <t>elc_spv_044</t>
+  </si>
+  <si>
+    <t>rez_spv_045</t>
+  </si>
+  <si>
+    <t>elc_spv_045</t>
+  </si>
+  <si>
+    <t>rez_spv_046</t>
+  </si>
+  <si>
+    <t>elc_spv_046</t>
+  </si>
+  <si>
+    <t>rez_spv_047</t>
+  </si>
+  <si>
+    <t>elc_spv_047</t>
+  </si>
+  <si>
+    <t>rez_spv_048</t>
+  </si>
+  <si>
+    <t>elc_spv_048</t>
+  </si>
+  <si>
+    <t>rez_spv_049</t>
+  </si>
+  <si>
+    <t>elc_spv_049</t>
+  </si>
+  <si>
+    <t>rez_spv_050</t>
+  </si>
+  <si>
+    <t>elc_spv_050</t>
+  </si>
+  <si>
+    <t>rez_spv_051</t>
+  </si>
+  <si>
+    <t>elc_spv_051</t>
+  </si>
+  <si>
+    <t>rez_spv_052</t>
+  </si>
+  <si>
+    <t>elc_spv_052</t>
+  </si>
+  <si>
+    <t>rez_spv_053</t>
+  </si>
+  <si>
+    <t>elc_spv_053</t>
+  </si>
+  <si>
+    <t>rez_spv_054</t>
+  </si>
+  <si>
+    <t>elc_spv_054</t>
+  </si>
+  <si>
+    <t>rez_spv_055</t>
+  </si>
+  <si>
+    <t>elc_spv_055</t>
+  </si>
+  <si>
+    <t>rez_spv_056</t>
+  </si>
+  <si>
+    <t>elc_spv_056</t>
+  </si>
+  <si>
+    <t>rez_spv_057</t>
+  </si>
+  <si>
+    <t>elc_spv_057</t>
+  </si>
+  <si>
+    <t>rez_spv_058</t>
+  </si>
+  <si>
+    <t>elc_spv_058</t>
+  </si>
+  <si>
+    <t>rez_spv_059</t>
+  </si>
+  <si>
+    <t>elc_spv_059</t>
+  </si>
+  <si>
+    <t>rez_spv_060</t>
+  </si>
+  <si>
+    <t>elc_spv_060</t>
+  </si>
+  <si>
+    <t>rez_spv_061</t>
+  </si>
+  <si>
+    <t>elc_spv_061</t>
+  </si>
+  <si>
+    <t>rez_spv_062</t>
+  </si>
+  <si>
+    <t>elc_spv_062</t>
+  </si>
+  <si>
+    <t>rez_spv_063</t>
+  </si>
+  <si>
+    <t>elc_spv_063</t>
+  </si>
+  <si>
+    <t>rez_spv_064</t>
+  </si>
+  <si>
+    <t>elc_spv_064</t>
+  </si>
+  <si>
+    <t>rez_spv_065</t>
+  </si>
+  <si>
+    <t>elc_spv_065</t>
+  </si>
+  <si>
+    <t>rez_spv_066</t>
+  </si>
+  <si>
+    <t>elc_spv_066</t>
+  </si>
+  <si>
+    <t>rez_spv_067</t>
+  </si>
+  <si>
+    <t>elc_spv_067</t>
+  </si>
+  <si>
+    <t>rez_spv_068</t>
+  </si>
+  <si>
+    <t>elc_spv_068</t>
+  </si>
+  <si>
+    <t>rez_spv_069</t>
+  </si>
+  <si>
+    <t>elc_spv_069</t>
+  </si>
+  <si>
+    <t>rez_spv_070</t>
+  </si>
+  <si>
+    <t>elc_spv_070</t>
+  </si>
+  <si>
+    <t>rez_spv_071</t>
+  </si>
+  <si>
+    <t>elc_spv_071</t>
+  </si>
+  <si>
+    <t>rez_spv_072</t>
+  </si>
+  <si>
+    <t>elc_spv_072</t>
+  </si>
+  <si>
+    <t>rez_spv_073</t>
+  </si>
+  <si>
+    <t>elc_spv_073</t>
+  </si>
+  <si>
+    <t>rez_spv_074</t>
+  </si>
+  <si>
+    <t>elc_spv_074</t>
+  </si>
+  <si>
+    <t>rez_spv_075</t>
+  </si>
+  <si>
+    <t>elc_spv_075</t>
+  </si>
+  <si>
+    <t>rez_spv_076</t>
+  </si>
+  <si>
+    <t>elc_spv_076</t>
+  </si>
+  <si>
+    <t>rez_spv_077</t>
+  </si>
+  <si>
+    <t>elc_spv_077</t>
+  </si>
+  <si>
+    <t>rez_spv_078</t>
+  </si>
+  <si>
+    <t>elc_spv_078</t>
+  </si>
+  <si>
+    <t>rez_spv_079</t>
+  </si>
+  <si>
+    <t>elc_spv_079</t>
+  </si>
+  <si>
+    <t>rez_spv_080</t>
+  </si>
+  <si>
+    <t>elc_spv_080</t>
+  </si>
+  <si>
+    <t>rez_spv_081</t>
+  </si>
+  <si>
+    <t>elc_spv_081</t>
+  </si>
+  <si>
+    <t>rez_spv_082</t>
+  </si>
+  <si>
+    <t>elc_spv_082</t>
+  </si>
+  <si>
+    <t>rez_spv_083</t>
+  </si>
+  <si>
+    <t>elc_spv_083</t>
+  </si>
+  <si>
+    <t>rez_spv_084</t>
+  </si>
+  <si>
+    <t>elc_spv_084</t>
+  </si>
+  <si>
+    <t>rez_spv_085</t>
+  </si>
+  <si>
+    <t>elc_spv_085</t>
+  </si>
+  <si>
+    <t>rez_spv_086</t>
+  </si>
+  <si>
+    <t>elc_spv_086</t>
+  </si>
+  <si>
+    <t>rez_spv_087</t>
+  </si>
+  <si>
+    <t>elc_spv_087</t>
+  </si>
+  <si>
+    <t>rez_spv_088</t>
+  </si>
+  <si>
+    <t>elc_spv_088</t>
+  </si>
+  <si>
+    <t>rez_spv_089</t>
+  </si>
+  <si>
+    <t>elc_spv_089</t>
+  </si>
+  <si>
+    <t>rez_spv_090</t>
+  </si>
+  <si>
+    <t>elc_spv_090</t>
+  </si>
+  <si>
+    <t>rez_spv_091</t>
+  </si>
+  <si>
+    <t>elc_spv_091</t>
+  </si>
+  <si>
+    <t>rez_spv_092</t>
+  </si>
+  <si>
+    <t>elc_spv_092</t>
+  </si>
+  <si>
+    <t>rez_spv_093</t>
+  </si>
+  <si>
+    <t>elc_spv_093</t>
+  </si>
+  <si>
+    <t>rez_spv_094</t>
+  </si>
+  <si>
+    <t>elc_spv_094</t>
+  </si>
+  <si>
+    <t>rez_spv_095</t>
+  </si>
+  <si>
+    <t>elc_spv_095</t>
+  </si>
+  <si>
+    <t>rez_spv_096</t>
+  </si>
+  <si>
+    <t>elc_spv_096</t>
+  </si>
+  <si>
+    <t>rez_spv_097</t>
+  </si>
+  <si>
+    <t>elc_spv_097</t>
+  </si>
+  <si>
+    <t>rez_spv_098</t>
+  </si>
+  <si>
+    <t>elc_spv_098</t>
+  </si>
+  <si>
+    <t>rez_spv_099</t>
+  </si>
+  <si>
+    <t>elc_spv_099</t>
+  </si>
+  <si>
+    <t>rez_spv_100</t>
+  </si>
+  <si>
+    <t>elc_spv_100</t>
+  </si>
+  <si>
+    <t>rez_spv_101</t>
+  </si>
+  <si>
+    <t>elc_spv_101</t>
+  </si>
+  <si>
+    <t>rez_spv_102</t>
+  </si>
+  <si>
+    <t>elc_spv_102</t>
+  </si>
+  <si>
+    <t>rez_spv_103</t>
+  </si>
+  <si>
+    <t>elc_spv_103</t>
+  </si>
+  <si>
+    <t>rez_spv_104</t>
+  </si>
+  <si>
+    <t>elc_spv_104</t>
+  </si>
+  <si>
+    <t>rez_spv_105</t>
+  </si>
+  <si>
+    <t>elc_spv_105</t>
+  </si>
+  <si>
+    <t>rez_spv_106</t>
+  </si>
+  <si>
+    <t>elc_spv_106</t>
+  </si>
+  <si>
+    <t>rez_spv_107</t>
+  </si>
+  <si>
+    <t>elc_spv_107</t>
+  </si>
+  <si>
+    <t>rez_spv_108</t>
+  </si>
+  <si>
+    <t>elc_spv_108</t>
+  </si>
+  <si>
+    <t>rez_spv_109</t>
+  </si>
+  <si>
+    <t>elc_spv_109</t>
+  </si>
+  <si>
+    <t>rez_spv_110</t>
+  </si>
+  <si>
+    <t>elc_spv_110</t>
+  </si>
+  <si>
+    <t>rez_spv_111</t>
+  </si>
+  <si>
+    <t>elc_spv_111</t>
+  </si>
+  <si>
+    <t>rez_spv_112</t>
+  </si>
+  <si>
+    <t>elc_spv_112</t>
   </si>
   <si>
     <t>rez_won_001</t>
@@ -5957,7 +5957,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88F0F5B4-89F6-4F2E-8B23-FBD0C54D6F08}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{096EF877-EBDD-47CC-A864-1C8955966A3C}">
   <dimension ref="B9:E805"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CAN_grids model - 2025-09-22 23:29
</commit_message>
<xml_diff>
--- a/VerveStacks_CAN_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_CAN_grids/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CAN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CE97F6B3-438B-4837-90B6-C9D9FF8C41B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1226B475-3459-4F7D-B333-EEBC128411E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5957,7 +5957,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{096EF877-EBDD-47CC-A864-1C8955966A3C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E214E29-3F12-456D-BF19-DB614CACF1AB}">
   <dimension ref="B9:E805"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>